<commit_message>
correction to previous commit
</commit_message>
<xml_diff>
--- a/VT_EE_ELC_V01.xlsx
+++ b/VT_EE_ELC_V01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B380FF01-0887-4980-AA73-9EA63544559A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48489F3D-34C0-42E2-BF33-7E3EA11F39B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" tabRatio="901" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6964,8 +6964,8 @@
         <v>ELCRESOL_VILJANDI00</v>
       </c>
       <c r="C29" s="21" t="str">
-        <f>$B$2&amp;RIGHT(Sector_Fuels_ELC!L13,3)</f>
-        <v>ELC</v>
+        <f>$B$2&amp;RIGHT(Sector_Fuels_ELC!L12,3)</f>
+        <v>ELCSOL</v>
       </c>
       <c r="D29" s="21" t="str">
         <f t="shared" si="0"/>
@@ -7022,8 +7022,8 @@
         <v>ELCRESOL_VORU00</v>
       </c>
       <c r="C30" s="21" t="str">
-        <f>$B$2&amp;RIGHT(Sector_Fuels_ELC!L14,3)</f>
-        <v>ELC</v>
+        <f>$B$2&amp;RIGHT(Sector_Fuels_ELC!L12,3)</f>
+        <v>ELCSOL</v>
       </c>
       <c r="D30" s="21" t="str">
         <f t="shared" si="0"/>
@@ -7080,8 +7080,8 @@
         <v>ELCRESOL_SAARE00</v>
       </c>
       <c r="C31" s="21" t="str">
-        <f>$B$2&amp;RIGHT(Sector_Fuels_ELC!L15,3)</f>
-        <v>ELCame</v>
+        <f>$B$2&amp;RIGHT(Sector_Fuels_ELC!L12,3)</f>
+        <v>ELCSOL</v>
       </c>
       <c r="D31" s="21" t="str">
         <f t="shared" si="0"/>
@@ -7138,8 +7138,8 @@
         <v>ELCRESOL_RAPLA00</v>
       </c>
       <c r="C32" s="21" t="str">
-        <f>$B$2&amp;RIGHT(Sector_Fuels_ELC!L16,3)</f>
-        <v>ELCame</v>
+        <f>$B$2&amp;RIGHT(Sector_Fuels_ELC!L12,3)</f>
+        <v>ELCSOL</v>
       </c>
       <c r="D32" s="21" t="str">
         <f t="shared" si="0"/>
@@ -7196,8 +7196,8 @@
         <v>ELCRESOL_LAANE00</v>
       </c>
       <c r="C33" s="21" t="str">
-        <f>$B$2&amp;RIGHT(Sector_Fuels_ELC!L17,3)</f>
-        <v>ELC</v>
+        <f>$B$2&amp;RIGHT(Sector_Fuels_ELC!L12,3)</f>
+        <v>ELCSOL</v>
       </c>
       <c r="D33" s="21" t="str">
         <f t="shared" si="0"/>
@@ -7254,8 +7254,8 @@
         <v>ELCRESOL_HIIU00</v>
       </c>
       <c r="C34" s="21" t="str">
-        <f>$B$2&amp;RIGHT(Sector_Fuels_ELC!L18,3)</f>
-        <v>ELCCOA</v>
+        <f>$B$2&amp;RIGHT(Sector_Fuels_ELC!L12,3)</f>
+        <v>ELCSOL</v>
       </c>
       <c r="D34" s="21" t="str">
         <f t="shared" si="0"/>

</xml_diff>

<commit_message>
FIx for previous commit
</commit_message>
<xml_diff>
--- a/VT_EE_ELC_V01.xlsx
+++ b/VT_EE_ELC_V01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64D5CBE5-9EAF-4A21-AC28-12BE82A69724}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44174599-D1CB-4906-88F2-EF4961911109}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="901" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="901" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EB1" sheetId="133" r:id="rId1"/>
@@ -7785,7 +7785,7 @@
     <row r="28" spans="1:26" x14ac:dyDescent="0.2">
       <c r="B28" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>ELCRESOL_SOPITOOTSI00</v>
+        <v>ELCREWON_SOPITOOTSI00</v>
       </c>
       <c r="C28" s="21" t="str">
         <f>$B$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)</f>
@@ -7826,8 +7826,8 @@
         <v>102</v>
       </c>
       <c r="V28" t="str">
-        <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$14,3)&amp;"_"&amp;Intra_areas!C3&amp;"00"</f>
-        <v>ELCRESOL_SOPITOOTSI00</v>
+        <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)&amp;"_"&amp;Intra_areas!C3&amp;"00"</f>
+        <v>ELCREWON_SOPITOOTSI00</v>
       </c>
       <c r="W28" t="str">
         <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V28,2)&amp;" in "&amp;Intra_areas!C3&amp;" - "&amp;'EB1'!$R$3</f>
@@ -7846,7 +7846,7 @@
     <row r="29" spans="1:26" x14ac:dyDescent="0.2">
       <c r="B29" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>ELCRESOL_SOPIPURTSE00</v>
+        <v>ELCREWON_SOPIPURTSE00</v>
       </c>
       <c r="C29" s="21" t="str">
         <f>$B$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)</f>
@@ -7887,8 +7887,8 @@
         <v>102</v>
       </c>
       <c r="V29" t="str">
-        <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$14,3)&amp;"_"&amp;Intra_areas!C4&amp;"00"</f>
-        <v>ELCRESOL_SOPIPURTSE00</v>
+        <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)&amp;"_"&amp;Intra_areas!C4&amp;"00"</f>
+        <v>ELCREWON_SOPIPURTSE00</v>
       </c>
       <c r="W29" t="str">
         <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V29,2)&amp;" in "&amp;Intra_areas!C4&amp;" - "&amp;'EB1'!$R$3</f>
@@ -7907,7 +7907,7 @@
     <row r="30" spans="1:26" x14ac:dyDescent="0.2">
       <c r="B30" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>ELCRESOL_OTHER00</v>
+        <v>ELCREWON_OTHER00</v>
       </c>
       <c r="C30" s="21" t="str">
         <f>$B$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)</f>
@@ -7948,8 +7948,8 @@
         <v>102</v>
       </c>
       <c r="V30" t="str">
-        <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$14,3)&amp;"_"&amp;Intra_areas!C5&amp;"00"</f>
-        <v>ELCRESOL_OTHER00</v>
+        <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)&amp;"_"&amp;Intra_areas!C5&amp;"00"</f>
+        <v>ELCREWON_OTHER00</v>
       </c>
       <c r="W30" t="str">
         <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V30,2)&amp;" in "&amp;Intra_areas!C5&amp;" - "&amp;'EB1'!$R$3</f>
@@ -7968,7 +7968,7 @@
     <row r="31" spans="1:26" x14ac:dyDescent="0.2">
       <c r="B31" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>ELCRESOL_SAARE00</v>
+        <v>ELCREWON_SAARE00</v>
       </c>
       <c r="C31" s="21" t="str">
         <f>$B$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)</f>
@@ -8009,8 +8009,8 @@
         <v>102</v>
       </c>
       <c r="V31" t="str">
-        <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$14,3)&amp;"_"&amp;Intra_areas!C6&amp;"00"</f>
-        <v>ELCRESOL_SAARE00</v>
+        <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)&amp;"_"&amp;Intra_areas!C6&amp;"00"</f>
+        <v>ELCREWON_SAARE00</v>
       </c>
       <c r="W31" t="str">
         <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V31,2)&amp;" in "&amp;Intra_areas!C6&amp;" - "&amp;'EB1'!$R$3</f>
@@ -8029,7 +8029,7 @@
     <row r="32" spans="1:26" x14ac:dyDescent="0.2">
       <c r="B32" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>ELCRESOL_LVIRU00</v>
+        <v>ELCREWON_LVIRU00</v>
       </c>
       <c r="C32" s="21" t="str">
         <f>$B$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)</f>
@@ -8070,8 +8070,8 @@
         <v>102</v>
       </c>
       <c r="V32" t="str">
-        <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$14,3)&amp;"_"&amp;Intra_areas!C7&amp;"00"</f>
-        <v>ELCRESOL_LVIRU00</v>
+        <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)&amp;"_"&amp;Intra_areas!C7&amp;"00"</f>
+        <v>ELCREWON_LVIRU00</v>
       </c>
       <c r="W32" t="str">
         <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V32,2)&amp;" in "&amp;Intra_areas!C7&amp;" - "&amp;'EB1'!$R$3</f>
@@ -8090,7 +8090,7 @@
     <row r="33" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B33" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>ELCRESOL_HARJU00</v>
+        <v>ELCREWON_HARJU00</v>
       </c>
       <c r="C33" s="21" t="str">
         <f>$B$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)</f>
@@ -8131,8 +8131,8 @@
         <v>102</v>
       </c>
       <c r="V33" t="str">
-        <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$14,3)&amp;"_"&amp;Intra_areas!C8&amp;"00"</f>
-        <v>ELCRESOL_HARJU00</v>
+        <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)&amp;"_"&amp;Intra_areas!C8&amp;"00"</f>
+        <v>ELCREWON_HARJU00</v>
       </c>
       <c r="W33" t="str">
         <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V33,2)&amp;" in "&amp;Intra_areas!C8&amp;" - "&amp;'EB1'!$R$3</f>
@@ -8151,7 +8151,7 @@
     <row r="34" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B34" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>ELCRESOL_LAANE00</v>
+        <v>ELCREWON_LAANE00</v>
       </c>
       <c r="C34" s="21" t="str">
         <f>$B$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)</f>
@@ -8192,8 +8192,8 @@
         <v>102</v>
       </c>
       <c r="V34" t="str">
-        <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$14,3)&amp;"_"&amp;Intra_areas!C9&amp;"00"</f>
-        <v>ELCRESOL_LAANE00</v>
+        <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)&amp;"_"&amp;Intra_areas!C9&amp;"00"</f>
+        <v>ELCREWON_LAANE00</v>
       </c>
       <c r="W34" t="str">
         <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V34,2)&amp;" in "&amp;Intra_areas!C9&amp;" - "&amp;'EB1'!$R$3</f>
@@ -8212,7 +8212,7 @@
     <row r="35" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B35" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>ELCRESOL_IVIRU00</v>
+        <v>ELCREWON_IVIRU00</v>
       </c>
       <c r="C35" s="21" t="str">
         <f>$B$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)</f>
@@ -8253,8 +8253,8 @@
         <v>102</v>
       </c>
       <c r="V35" t="str">
-        <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$14,3)&amp;"_"&amp;Intra_areas!C10&amp;"00"</f>
-        <v>ELCRESOL_IVIRU00</v>
+        <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)&amp;"_"&amp;Intra_areas!C10&amp;"00"</f>
+        <v>ELCREWON_IVIRU00</v>
       </c>
       <c r="W35" t="str">
         <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V35,2)&amp;" in "&amp;Intra_areas!C10&amp;" - "&amp;'EB1'!$R$3</f>
@@ -8273,7 +8273,7 @@
     <row r="36" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B36" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>ELCRESOL_PARNU00</v>
+        <v>ELCREWON_PARNU00</v>
       </c>
       <c r="C36" s="21" t="str">
         <f>$B$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)</f>
@@ -8314,8 +8314,8 @@
         <v>102</v>
       </c>
       <c r="V36" t="str">
-        <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$14,3)&amp;"_"&amp;Intra_areas!C11&amp;"00"</f>
-        <v>ELCRESOL_PARNU00</v>
+        <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)&amp;"_"&amp;Intra_areas!C11&amp;"00"</f>
+        <v>ELCREWON_PARNU00</v>
       </c>
       <c r="W36" t="str">
         <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V36,2)&amp;" in "&amp;Intra_areas!C11&amp;" - "&amp;'EB1'!$R$3</f>

</xml_diff>

<commit_message>
Adding a missing link for oil shale PPs
</commit_message>
<xml_diff>
--- a/VT_EE_ELC_V01.xlsx
+++ b/VT_EE_ELC_V01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E03520AE-64B2-4014-B4AF-177EAA8A7857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13E6EBA0-8112-4F88-87F6-AE9F44E93B84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" tabRatio="901" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" tabRatio="901" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EB1" sheetId="133" r:id="rId1"/>
@@ -6328,6 +6328,26 @@
         <v>30</v>
       </c>
     </row>
+    <row r="36" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B36" s="21" t="str">
+        <f>Sector_Fuels_ELC!L33</f>
+        <v>FTE-ELCSHL</v>
+      </c>
+      <c r="C36" t="str">
+        <f>RIGHT(D36,3)</f>
+        <v>SHL</v>
+      </c>
+      <c r="D36" s="21" t="str">
+        <f>L16</f>
+        <v>ELCSHL</v>
+      </c>
+      <c r="G36" s="61">
+        <v>1</v>
+      </c>
+      <c r="H36" s="62">
+        <v>30</v>
+      </c>
+    </row>
     <row r="40" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B40" s="43"/>
       <c r="C40" s="1" t="s">

</xml_diff>

<commit_message>
Attempt on turning off capacity's linear decomissioning
</commit_message>
<xml_diff>
--- a/VT_EE_ELC_V01.xlsx
+++ b/VT_EE_ELC_V01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA1D19DA-9F10-4BFF-839A-165D5F18F9C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B82AF2F4-6681-4C4E-B585-55D05881DF4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" tabRatio="901" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="901" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EB1" sheetId="133" r:id="rId1"/>
@@ -786,9 +786,10 @@
     <author>Gary Goldstein</author>
     <author>Amit Kanudia</author>
     <author>Maurizio Gargiulo</author>
+    <author>Kristopher Raik</author>
   </authors>
   <commentList>
-    <comment ref="T3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000001000000}">
+    <comment ref="U3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000001000000}">
       <text>
         <r>
           <rPr>
@@ -902,7 +903,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Y3" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0300-000002000000}">
+    <comment ref="Z3" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0300-000002000000}">
       <text>
         <r>
           <rPr>
@@ -928,7 +929,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z3" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0300-000003000000}">
+    <comment ref="AA3" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0300-000003000000}">
       <text>
         <r>
           <rPr>
@@ -1001,7 +1002,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AA3" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0300-000004000000}">
+    <comment ref="AB3" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0300-000004000000}">
       <text>
         <r>
           <rPr>
@@ -1054,7 +1055,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB3" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0300-000005000000}">
+    <comment ref="AC3" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0300-000005000000}">
       <text>
         <r>
           <rPr>
@@ -1087,7 +1088,33 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z9" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0300-000006000000}">
+    <comment ref="G9" authorId="3" shapeId="0" xr:uid="{4CC104A8-D70F-4C07-9649-7404261279B2}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+            <charset val="186"/>
+          </rPr>
+          <t>Kristopher Raik:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+            <charset val="186"/>
+          </rPr>
+          <t xml:space="preserve">
+use PASTI (2024) is constant over technical life</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AA9" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0300-000006000000}">
       <text>
         <r>
           <rPr>
@@ -1180,7 +1207,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AA9" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0300-000007000000}">
+    <comment ref="AB9" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0300-000007000000}">
       <text>
         <r>
           <rPr>
@@ -1205,7 +1232,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB9" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0300-000008000000}">
+    <comment ref="AC9" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0300-000008000000}">
       <text>
         <r>
           <rPr>
@@ -1268,7 +1295,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T10" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0300-000009000000}">
+    <comment ref="U10" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0300-000009000000}">
       <text>
         <r>
           <rPr>
@@ -1508,6 +1535,32 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve"> (Heating Plant)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I12" authorId="3" shapeId="0" xr:uid="{49F8970F-654D-4377-A47F-D4881BFD24ED}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+            <charset val="186"/>
+          </rPr>
+          <t>Kristopher Raik:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+            <charset val="186"/>
+          </rPr>
+          <t xml:space="preserve">
+Variable == 2 means that. So new capacity = 0</t>
         </r>
       </text>
     </comment>
@@ -2280,7 +2333,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="610" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="611" uniqueCount="207">
   <si>
     <t>CommName</t>
   </si>
@@ -2895,6 +2948,12 @@
   </si>
   <si>
     <t>Total CO2</t>
+  </si>
+  <si>
+    <t>NCAP_BND~0</t>
+  </si>
+  <si>
+    <t>PASTI~2025</t>
   </si>
 </sst>
 </file>
@@ -2909,7 +2968,7 @@
     <numFmt numFmtId="167" formatCode="0.0000"/>
     <numFmt numFmtId="168" formatCode="\Te\x\t"/>
   </numFmts>
-  <fonts count="28" x14ac:knownFonts="1">
+  <fonts count="30" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -2917,6 +2976,8 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
+      <charset val="186"/>
     </font>
     <font>
       <sz val="10"/>
@@ -2979,6 +3040,8 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
+      <charset val="186"/>
     </font>
     <font>
       <sz val="11"/>
@@ -3084,6 +3147,21 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+      <charset val="186"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+      <charset val="186"/>
     </font>
   </fonts>
   <fills count="18">
@@ -3881,13 +3959,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>17</xdr:col>
+      <xdr:col>18</xdr:col>
       <xdr:colOff>871640</xdr:colOff>
       <xdr:row>63</xdr:row>
       <xdr:rowOff>120128</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
+      <xdr:col>25</xdr:col>
       <xdr:colOff>692699</xdr:colOff>
       <xdr:row>71</xdr:row>
       <xdr:rowOff>115715</xdr:rowOff>
@@ -6894,7 +6972,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="B1:AB65529"/>
+  <dimension ref="B1:AC65529"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3" style="21" customWidth="1"/>
@@ -6903,29 +6981,30 @@
     <col min="4" max="4" width="11.28515625" style="21" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="12" style="21" bestFit="1" customWidth="1"/>
     <col min="7" max="8" width="13" style="21" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.85546875" style="21" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.140625" style="21" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10" style="21" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="8.85546875" style="21" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15" style="21" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.28515625" style="21" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="2" style="21" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.5703125" style="21" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="2.140625" style="21" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="57.7109375" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="6.28515625" customWidth="1"/>
-    <col min="25" max="25" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="15" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="29" max="16384" width="8.85546875" style="21"/>
+    <col min="9" max="9" width="13" style="21" customWidth="1"/>
+    <col min="10" max="10" width="8.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.140625" style="21" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10" style="21" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="8.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15" style="21" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.28515625" style="21" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="2" style="21" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.5703125" style="21" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="2.140625" style="21" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="57.7109375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="6.28515625" customWidth="1"/>
+    <col min="26" max="26" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="15" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="30" max="16384" width="8.85546875" style="21"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:28" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:29" ht="30" x14ac:dyDescent="0.25">
       <c r="B1" s="20" t="s">
         <v>65</v>
       </c>
@@ -6947,8 +7026,9 @@
       <c r="H1" s="20" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="2" spans="2:28" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="I1" s="20"/>
+    </row>
+    <row r="2" spans="2:29" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B2" s="10" t="str">
         <f>'EB1'!B6</f>
         <v>ELC</v>
@@ -6974,48 +7054,49 @@
       <c r="H2" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="T2" s="84" t="s">
+      <c r="I2" s="10"/>
+      <c r="U2" s="84" t="s">
         <v>14</v>
       </c>
-      <c r="U2" s="84"/>
-      <c r="V2" s="85"/>
+      <c r="V2" s="84"/>
       <c r="W2" s="85"/>
       <c r="X2" s="85"/>
       <c r="Y2" s="85"/>
       <c r="Z2" s="85"/>
       <c r="AA2" s="85"/>
       <c r="AB2" s="85"/>
-    </row>
-    <row r="3" spans="2:28" x14ac:dyDescent="0.2">
-      <c r="T3" s="86" t="s">
+      <c r="AC2" s="85"/>
+    </row>
+    <row r="3" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="U3" s="86" t="s">
         <v>7</v>
       </c>
-      <c r="U3" s="87" t="s">
+      <c r="V3" s="87" t="s">
         <v>30</v>
       </c>
-      <c r="V3" s="86" t="s">
+      <c r="W3" s="86" t="s">
         <v>0</v>
       </c>
-      <c r="W3" s="86" t="s">
+      <c r="X3" s="86" t="s">
         <v>3</v>
       </c>
-      <c r="X3" s="86" t="s">
+      <c r="Y3" s="86" t="s">
         <v>4</v>
       </c>
-      <c r="Y3" s="86" t="s">
+      <c r="Z3" s="86" t="s">
         <v>8</v>
       </c>
-      <c r="Z3" s="86" t="s">
+      <c r="AA3" s="86" t="s">
         <v>9</v>
       </c>
-      <c r="AA3" s="86" t="s">
+      <c r="AB3" s="86" t="s">
         <v>10</v>
       </c>
-      <c r="AB3" s="86" t="s">
+      <c r="AC3" s="86" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="2:28" ht="24" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:29" ht="24" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="25" t="s">
         <v>107</v>
       </c>
@@ -7032,36 +7113,37 @@
         <v>121</v>
       </c>
       <c r="H4" s="9"/>
-      <c r="K4" s="9"/>
-      <c r="T4" s="88" t="s">
+      <c r="I4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="U4" s="88" t="s">
         <v>35</v>
       </c>
-      <c r="U4" s="88" t="s">
+      <c r="V4" s="88" t="s">
         <v>31</v>
       </c>
-      <c r="V4" s="88" t="s">
+      <c r="W4" s="88" t="s">
         <v>26</v>
       </c>
-      <c r="W4" s="88" t="s">
+      <c r="X4" s="88" t="s">
         <v>27</v>
       </c>
-      <c r="X4" s="88" t="s">
+      <c r="Y4" s="88" t="s">
         <v>4</v>
       </c>
-      <c r="Y4" s="88" t="s">
+      <c r="Z4" s="88" t="s">
         <v>38</v>
       </c>
-      <c r="Z4" s="88" t="s">
+      <c r="AA4" s="88" t="s">
         <v>39</v>
       </c>
-      <c r="AA4" s="88" t="s">
+      <c r="AB4" s="88" t="s">
         <v>28</v>
       </c>
-      <c r="AB4" s="88" t="s">
+      <c r="AC4" s="88" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="2:28" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:29" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B5" s="24" t="s">
         <v>113</v>
       </c>
@@ -7078,58 +7160,59 @@
         <v>85</v>
       </c>
       <c r="H5" s="9"/>
-      <c r="K5" s="9"/>
-      <c r="T5" s="85" t="s">
+      <c r="I5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="U5" s="85" t="s">
         <v>64</v>
       </c>
-      <c r="U5" s="89"/>
-      <c r="V5" s="85" t="s">
+      <c r="V5" s="89"/>
+      <c r="W5" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="W5" s="85" t="str">
+      <c r="X5" s="85" t="str">
         <f>'EB1'!$W$3</f>
         <v>Electricity</v>
       </c>
-      <c r="X5" s="85" t="str">
+      <c r="Y5" s="85" t="str">
         <f>$E$2</f>
         <v>PJ</v>
       </c>
-      <c r="Y5" s="85"/>
-      <c r="Z5" s="85" t="s">
+      <c r="Z5" s="85"/>
+      <c r="AA5" s="85" t="s">
         <v>116</v>
       </c>
-      <c r="AA5" s="85"/>
-      <c r="AB5" s="85" t="s">
+      <c r="AB5" s="85"/>
+      <c r="AC5" s="85" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="6" spans="2:28" x14ac:dyDescent="0.2">
-      <c r="T6" s="89" t="s">
+    <row r="6" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="U6" s="89" t="s">
         <v>88</v>
       </c>
-      <c r="U6" s="89"/>
-      <c r="V6" s="89" t="str">
+      <c r="V6" s="89"/>
+      <c r="W6" s="89" t="str">
         <f>$B$2&amp;'EB1'!$C$15</f>
         <v>ELCCO2</v>
       </c>
-      <c r="W6" s="89" t="str">
+      <c r="X6" s="89" t="str">
         <f>$C$2&amp;" "&amp;'EB1'!$C$16</f>
         <v>Electricity Plants Carbon dioxide</v>
       </c>
-      <c r="X6" s="89" t="str">
+      <c r="Y6" s="89" t="str">
         <f>'EB1'!$AC$2</f>
         <v>kt</v>
       </c>
-      <c r="Y6" s="89"/>
       <c r="Z6" s="89"/>
       <c r="AA6" s="89"/>
       <c r="AB6" s="89"/>
-    </row>
-    <row r="7" spans="2:28" x14ac:dyDescent="0.2">
-      <c r="T7" s="2"/>
+      <c r="AC6" s="89"/>
+    </row>
+    <row r="7" spans="2:29" x14ac:dyDescent="0.2">
       <c r="U7" s="2"/>
-    </row>
-    <row r="8" spans="2:28" x14ac:dyDescent="0.2">
+      <c r="V7" s="2"/>
+    </row>
+    <row r="8" spans="2:29" x14ac:dyDescent="0.2">
       <c r="D8" s="4" t="s">
         <v>13</v>
       </c>
@@ -7138,22 +7221,23 @@
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
-      <c r="L8" s="5"/>
+      <c r="J8" s="4"/>
       <c r="M8" s="5"/>
-      <c r="N8" s="3"/>
-      <c r="T8" s="84" t="s">
+      <c r="N8" s="5"/>
+      <c r="O8" s="3"/>
+      <c r="U8" s="84" t="s">
         <v>15</v>
       </c>
-      <c r="U8" s="84"/>
-      <c r="V8" s="85"/>
+      <c r="V8" s="84"/>
       <c r="W8" s="85"/>
       <c r="X8" s="85"/>
       <c r="Y8" s="85"/>
       <c r="Z8" s="85"/>
       <c r="AA8" s="85"/>
       <c r="AB8" s="85"/>
-    </row>
-    <row r="9" spans="2:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AC8" s="85"/>
+    </row>
+    <row r="9" spans="2:29" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="17" t="s">
         <v>1</v>
       </c>
@@ -7170,69 +7254,72 @@
         <v>160</v>
       </c>
       <c r="G9" s="67" t="s">
-        <v>122</v>
+        <v>206</v>
       </c>
       <c r="H9" s="67" t="s">
         <v>144</v>
       </c>
       <c r="I9" s="67" t="s">
+        <v>205</v>
+      </c>
+      <c r="J9" s="67" t="s">
         <v>73</v>
       </c>
-      <c r="J9" s="67" t="s">
+      <c r="K9" s="67" t="s">
         <v>162</v>
       </c>
-      <c r="K9" s="67" t="s">
+      <c r="L9" s="67" t="s">
         <v>157</v>
       </c>
-      <c r="L9" s="67" t="s">
+      <c r="M9" s="67" t="s">
         <v>72</v>
       </c>
-      <c r="M9" s="67" t="s">
+      <c r="N9" s="67" t="s">
         <v>103</v>
       </c>
-      <c r="N9" s="67" t="s">
+      <c r="O9" s="67" t="s">
         <v>70</v>
       </c>
-      <c r="O9" s="67" t="s">
+      <c r="P9" s="67" t="s">
         <v>156</v>
       </c>
-      <c r="P9" s="67" t="s">
+      <c r="Q9" s="67" t="s">
         <v>117</v>
       </c>
-      <c r="Q9" s="23"/>
-      <c r="R9" s="80" t="s">
+      <c r="R9" s="23"/>
+      <c r="S9" s="80" t="s">
         <v>115</v>
       </c>
-      <c r="S9" s="27"/>
-      <c r="T9" s="86" t="s">
+      <c r="T9" s="27"/>
+      <c r="U9" s="86" t="s">
         <v>11</v>
       </c>
-      <c r="U9" s="87" t="s">
+      <c r="V9" s="87" t="s">
         <v>30</v>
       </c>
-      <c r="V9" s="86" t="s">
+      <c r="W9" s="86" t="s">
         <v>1</v>
       </c>
-      <c r="W9" s="86" t="s">
+      <c r="X9" s="86" t="s">
         <v>2</v>
       </c>
-      <c r="X9" s="86" t="s">
+      <c r="Y9" s="86" t="s">
         <v>16</v>
       </c>
-      <c r="Y9" s="86" t="s">
+      <c r="Z9" s="86" t="s">
         <v>17</v>
       </c>
-      <c r="Z9" s="86" t="s">
+      <c r="AA9" s="86" t="s">
         <v>18</v>
       </c>
-      <c r="AA9" s="86" t="s">
+      <c r="AB9" s="86" t="s">
         <v>19</v>
       </c>
-      <c r="AB9" s="86" t="s">
+      <c r="AC9" s="86" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="2:28" ht="23.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:29" ht="23.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B10" s="15" t="s">
         <v>37</v>
       </c>
@@ -7254,63 +7341,64 @@
       <c r="H10" s="73" t="s">
         <v>119</v>
       </c>
-      <c r="I10" s="15" t="s">
+      <c r="I10" s="15"/>
+      <c r="J10" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="J10" s="73" t="s">
+      <c r="K10" s="73" t="s">
         <v>82</v>
       </c>
-      <c r="K10" s="15" t="s">
+      <c r="L10" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="L10" s="15" t="s">
+      <c r="M10" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="M10" s="15" t="s">
+      <c r="N10" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="N10" s="15" t="s">
+      <c r="O10" s="15" t="s">
         <v>155</v>
       </c>
-      <c r="O10" s="15" t="s">
+      <c r="P10" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="P10" s="15" t="s">
+      <c r="Q10" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="R10" s="30" t="s">
+      <c r="S10" s="30" t="s">
         <v>104</v>
       </c>
-      <c r="S10" s="28"/>
-      <c r="T10" s="88" t="s">
+      <c r="T10" s="28"/>
+      <c r="U10" s="88" t="s">
         <v>36</v>
       </c>
-      <c r="U10" s="88" t="s">
+      <c r="V10" s="88" t="s">
         <v>31</v>
       </c>
-      <c r="V10" s="88" t="s">
+      <c r="W10" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="W10" s="88" t="s">
+      <c r="X10" s="88" t="s">
         <v>22</v>
       </c>
-      <c r="X10" s="88" t="s">
+      <c r="Y10" s="88" t="s">
         <v>23</v>
       </c>
-      <c r="Y10" s="88" t="s">
+      <c r="Z10" s="88" t="s">
         <v>24</v>
       </c>
-      <c r="Z10" s="88" t="s">
+      <c r="AA10" s="88" t="s">
         <v>41</v>
       </c>
-      <c r="AA10" s="88" t="s">
+      <c r="AB10" s="88" t="s">
         <v>40</v>
       </c>
-      <c r="AB10" s="88" t="s">
+      <c r="AC10" s="88" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="2:28" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:29" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B11" s="14" t="s">
         <v>76</v>
       </c>
@@ -7332,35 +7420,35 @@
         <f>$F$2</f>
         <v>GW</v>
       </c>
-      <c r="I11" s="13"/>
-      <c r="J11" s="68"/>
-      <c r="K11" s="13" t="str">
-        <f>$G$2&amp;"/"&amp;$F$2</f>
-        <v>M€2025/GW</v>
-      </c>
+      <c r="I11" s="68"/>
+      <c r="J11" s="13"/>
+      <c r="K11" s="68"/>
       <c r="L11" s="13" t="str">
         <f>$G$2&amp;"/"&amp;$F$2</f>
         <v>M€2025/GW</v>
       </c>
       <c r="M11" s="13" t="str">
+        <f>$G$2&amp;"/"&amp;$F$2</f>
+        <v>M€2025/GW</v>
+      </c>
+      <c r="N11" s="13" t="str">
         <f>$G$2&amp;"/"&amp;$E$2</f>
         <v>M€2025/PJ</v>
       </c>
-      <c r="N11" s="13" t="s">
+      <c r="O11" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="O11" s="13" t="s">
+      <c r="P11" s="13" t="s">
         <v>193</v>
       </c>
-      <c r="P11" s="13"/>
-      <c r="R11" s="81" t="s">
+      <c r="Q11" s="13"/>
+      <c r="S11" s="81" t="s">
         <v>120</v>
       </c>
-      <c r="S11" s="28"/>
-      <c r="T11" s="88" t="s">
+      <c r="T11" s="28"/>
+      <c r="U11" s="88" t="s">
         <v>71</v>
       </c>
-      <c r="U11" s="88"/>
       <c r="V11" s="88"/>
       <c r="W11" s="88"/>
       <c r="X11" s="88"/>
@@ -7368,10 +7456,11 @@
       <c r="Z11" s="88"/>
       <c r="AA11" s="88"/>
       <c r="AB11" s="88"/>
-    </row>
-    <row r="12" spans="2:28" x14ac:dyDescent="0.2">
+      <c r="AC11" s="88"/>
+    </row>
+    <row r="12" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B12" s="21" t="str">
-        <f>V12</f>
+        <f>W12</f>
         <v>ELCREHYD00</v>
       </c>
       <c r="C12" s="21" t="str">
@@ -7379,7 +7468,7 @@
         <v>ELCHYD</v>
       </c>
       <c r="D12" s="21" t="str">
-        <f t="shared" ref="D12:D48" si="0">$V$5</f>
+        <f t="shared" ref="D12:D48" si="0">$W$5</f>
         <v>ELC</v>
       </c>
       <c r="E12" s="42"/>
@@ -7388,55 +7477,58 @@
         <v>8.0000000000000002E-3</v>
       </c>
       <c r="H12" s="83"/>
-      <c r="I12" s="63">
+      <c r="I12" s="7">
+        <v>2</v>
+      </c>
+      <c r="J12" s="63">
         <v>1</v>
       </c>
-      <c r="J12" s="63">
+      <c r="K12" s="63">
         <v>0.5</v>
       </c>
-      <c r="K12" s="63"/>
-      <c r="L12" s="42"/>
-      <c r="M12" s="63"/>
-      <c r="N12" s="42"/>
-      <c r="O12" s="64">
+      <c r="L12" s="63"/>
+      <c r="M12" s="42"/>
+      <c r="N12" s="63"/>
+      <c r="O12" s="42"/>
+      <c r="P12" s="64">
         <v>8.76</v>
       </c>
-      <c r="P12" s="65">
+      <c r="Q12" s="65">
         <v>0.5</v>
       </c>
-      <c r="R12" s="26">
-        <f>(E12+F12)*$J12*$O12</f>
+      <c r="S12" s="26">
+        <f>(E12+F12)*$K12*$P12</f>
         <v>0</v>
       </c>
-      <c r="S12" s="29"/>
-      <c r="T12" s="89" t="s">
+      <c r="T12" s="29"/>
+      <c r="U12" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="U12" s="89"/>
-      <c r="V12" s="89" t="str">
+      <c r="V12" s="89"/>
+      <c r="W12" s="89" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$10,3)&amp;"00"</f>
         <v>ELCREHYD00</v>
       </c>
-      <c r="W12" s="89" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V12,2)&amp;" - "&amp;'EB1'!P3</f>
+      <c r="X12" s="89" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W12,2)&amp;" - "&amp;'EB1'!P3</f>
         <v>Power Plants Existing00 - Hydro power</v>
       </c>
-      <c r="X12" t="s">
+      <c r="Y12" t="s">
         <v>180</v>
       </c>
-      <c r="Y12" s="89" t="str">
-        <f t="shared" ref="Y12" si="1">$F$2</f>
+      <c r="Z12" s="89" t="str">
+        <f t="shared" ref="Z12" si="1">$F$2</f>
         <v>GW</v>
       </c>
-      <c r="Z12" t="s">
+      <c r="AA12" t="s">
         <v>116</v>
       </c>
-      <c r="AA12" s="89"/>
       <c r="AB12" s="89"/>
-    </row>
-    <row r="13" spans="2:28" x14ac:dyDescent="0.2">
+      <c r="AC12" s="89"/>
+    </row>
+    <row r="13" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B13" s="21" t="str">
-        <f>V13</f>
+        <f>W13</f>
         <v>ELCRESOL_PARNU00</v>
       </c>
       <c r="C13" s="21" t="str">
@@ -7450,54 +7542,57 @@
       <c r="G13">
         <v>0.24199999999999999</v>
       </c>
-      <c r="I13" s="93">
+      <c r="I13" s="7">
+        <v>2</v>
+      </c>
+      <c r="J13" s="93">
         <v>1</v>
       </c>
-      <c r="J13" s="63">
+      <c r="K13" s="63">
         <v>0.3</v>
       </c>
-      <c r="K13" s="7">
+      <c r="L13" s="7">
         <v>1018</v>
       </c>
-      <c r="L13" s="83">
+      <c r="M13" s="83">
         <v>16.064040000000002</v>
       </c>
-      <c r="M13" s="83">
+      <c r="N13" s="83">
         <v>0</v>
       </c>
-      <c r="N13" s="21">
+      <c r="O13" s="21">
         <v>35</v>
       </c>
-      <c r="O13" s="64">
+      <c r="P13" s="64">
         <v>8.76</v>
       </c>
-      <c r="P13" s="74">
+      <c r="Q13" s="74">
         <v>0.1461854238754417</v>
       </c>
-      <c r="T13" s="89" t="s">
+      <c r="U13" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V13" s="89" t="str">
+      <c r="W13" s="89" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$14,3)&amp;"_"&amp;Intra_areas!B3&amp;"00"</f>
         <v>ELCRESOL_PARNU00</v>
       </c>
-      <c r="W13" s="89" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V13,2)&amp;" in "&amp;Intra_areas!B3&amp;" - "&amp;'EB1'!$T$3</f>
+      <c r="X13" s="89" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W13,2)&amp;" in "&amp;Intra_areas!B3&amp;" - "&amp;'EB1'!$T$3</f>
         <v>Power Plants Existing00 in PARNU - Solar energy</v>
       </c>
-      <c r="X13" t="s">
+      <c r="Y13" t="s">
         <v>180</v>
       </c>
-      <c r="Y13" t="s">
+      <c r="Z13" t="s">
         <v>101</v>
       </c>
-      <c r="Z13" t="s">
+      <c r="AA13" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="14" spans="2:28" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B14" s="21" t="str">
-        <f t="shared" ref="B14:B37" si="2">V14</f>
+        <f t="shared" ref="B14:B37" si="2">W14</f>
         <v>ELCRESOL_TARTU00</v>
       </c>
       <c r="C14" s="21" t="str">
@@ -7511,53 +7606,56 @@
       <c r="G14">
         <v>0.108</v>
       </c>
-      <c r="I14" s="93">
+      <c r="I14" s="7">
+        <v>2</v>
+      </c>
+      <c r="J14" s="93">
         <v>1</v>
       </c>
-      <c r="J14" s="63">
+      <c r="K14" s="63">
         <v>0.3</v>
       </c>
-      <c r="K14" s="7">
+      <c r="L14" s="7">
         <v>1018</v>
       </c>
-      <c r="L14" s="83">
+      <c r="M14" s="83">
         <v>16.064040000000002</v>
       </c>
-      <c r="M14" s="83">
+      <c r="N14" s="83">
         <v>0</v>
       </c>
-      <c r="N14" s="21">
+      <c r="O14" s="21">
         <v>35</v>
       </c>
-      <c r="O14" s="64">
+      <c r="P14" s="64">
         <v>8.76</v>
       </c>
-      <c r="P14" s="74">
+      <c r="Q14" s="74">
         <v>0.1461854238754417</v>
       </c>
-      <c r="R14" s="79"/>
-      <c r="T14" s="89" t="s">
+      <c r="S14" s="79"/>
+      <c r="U14" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V14" s="89" t="str">
+      <c r="W14" s="89" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$14,3)&amp;"_"&amp;Intra_areas!B4&amp;"00"</f>
         <v>ELCRESOL_TARTU00</v>
       </c>
-      <c r="W14" s="89" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V14,2)&amp;" in "&amp;Intra_areas!B4&amp;" - "&amp;'EB1'!$T$3</f>
+      <c r="X14" s="89" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W14,2)&amp;" in "&amp;Intra_areas!B4&amp;" - "&amp;'EB1'!$T$3</f>
         <v>Power Plants Existing00 in TARTU - Solar energy</v>
       </c>
-      <c r="X14" t="s">
+      <c r="Y14" t="s">
         <v>180</v>
       </c>
-      <c r="Y14" t="s">
+      <c r="Z14" t="s">
         <v>101</v>
       </c>
-      <c r="Z14" t="s">
+      <c r="AA14" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="15" spans="2:28" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B15" s="21" t="str">
         <f t="shared" si="2"/>
         <v>ELCRESOL_LVIRU00</v>
@@ -7573,53 +7671,56 @@
       <c r="G15">
         <v>0.13200000000000001</v>
       </c>
-      <c r="I15" s="93">
+      <c r="I15" s="7">
+        <v>2</v>
+      </c>
+      <c r="J15" s="93">
         <v>1</v>
       </c>
-      <c r="J15" s="63">
+      <c r="K15" s="63">
         <v>0.3</v>
       </c>
-      <c r="K15" s="7">
+      <c r="L15" s="7">
         <v>1018</v>
       </c>
-      <c r="L15" s="83">
+      <c r="M15" s="83">
         <v>16.064040000000002</v>
       </c>
-      <c r="M15" s="83">
+      <c r="N15" s="83">
         <v>0</v>
       </c>
-      <c r="N15" s="21">
+      <c r="O15" s="21">
         <v>35</v>
       </c>
-      <c r="O15" s="64">
+      <c r="P15" s="64">
         <v>8.76</v>
       </c>
-      <c r="P15" s="74">
+      <c r="Q15" s="74">
         <v>0.14867925344692126</v>
       </c>
-      <c r="R15" s="79"/>
-      <c r="T15" s="89" t="s">
+      <c r="S15" s="79"/>
+      <c r="U15" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V15" s="89" t="str">
+      <c r="W15" s="89" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$14,3)&amp;"_"&amp;Intra_areas!B5&amp;"00"</f>
         <v>ELCRESOL_LVIRU00</v>
       </c>
-      <c r="W15" s="89" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V15,2)&amp;" in "&amp;Intra_areas!B5&amp;" - "&amp;'EB1'!$T$3</f>
+      <c r="X15" s="89" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W15,2)&amp;" in "&amp;Intra_areas!B5&amp;" - "&amp;'EB1'!$T$3</f>
         <v>Power Plants Existing00 in LVIRU - Solar energy</v>
       </c>
-      <c r="X15" t="s">
+      <c r="Y15" t="s">
         <v>180</v>
       </c>
-      <c r="Y15" t="s">
+      <c r="Z15" t="s">
         <v>101</v>
       </c>
-      <c r="Z15" t="s">
+      <c r="AA15" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="16" spans="2:28" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B16" s="21" t="str">
         <f t="shared" si="2"/>
         <v>ELCRESOL_IVIRU00</v>
@@ -7635,53 +7736,56 @@
       <c r="G16">
         <v>7.8E-2</v>
       </c>
-      <c r="I16" s="93">
+      <c r="I16" s="7">
+        <v>2</v>
+      </c>
+      <c r="J16" s="93">
         <v>1</v>
       </c>
-      <c r="J16" s="63">
+      <c r="K16" s="63">
         <v>0.3</v>
       </c>
-      <c r="K16" s="7">
+      <c r="L16" s="7">
         <v>1018</v>
       </c>
-      <c r="L16" s="83">
+      <c r="M16" s="83">
         <v>16.064040000000002</v>
       </c>
-      <c r="M16" s="83">
+      <c r="N16" s="83">
         <v>0</v>
       </c>
-      <c r="N16" s="21">
+      <c r="O16" s="21">
         <v>35</v>
       </c>
-      <c r="O16" s="64">
+      <c r="P16" s="64">
         <v>8.76</v>
       </c>
-      <c r="P16" s="74">
+      <c r="Q16" s="74">
         <v>0.14701259708091721</v>
       </c>
-      <c r="R16" s="79"/>
-      <c r="T16" s="89" t="s">
+      <c r="S16" s="79"/>
+      <c r="U16" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V16" s="89" t="str">
+      <c r="W16" s="89" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$14,3)&amp;"_"&amp;Intra_areas!B6&amp;"00"</f>
         <v>ELCRESOL_IVIRU00</v>
       </c>
-      <c r="W16" s="89" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V16,2)&amp;" in "&amp;Intra_areas!B6&amp;" - "&amp;'EB1'!$T$3</f>
+      <c r="X16" s="89" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W16,2)&amp;" in "&amp;Intra_areas!B6&amp;" - "&amp;'EB1'!$T$3</f>
         <v>Power Plants Existing00 in IVIRU - Solar energy</v>
       </c>
-      <c r="X16" t="s">
+      <c r="Y16" t="s">
         <v>180</v>
       </c>
-      <c r="Y16" t="s">
+      <c r="Z16" t="s">
         <v>101</v>
       </c>
-      <c r="Z16" t="s">
+      <c r="AA16" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="17" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B17" s="21" t="str">
         <f t="shared" si="2"/>
         <v>ELCRESOL_JARVA00</v>
@@ -7697,53 +7801,56 @@
       <c r="G17">
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="I17" s="93">
+      <c r="I17" s="7">
+        <v>2</v>
+      </c>
+      <c r="J17" s="93">
         <v>1</v>
       </c>
-      <c r="J17" s="63">
+      <c r="K17" s="63">
         <v>0.3</v>
       </c>
-      <c r="K17" s="7">
+      <c r="L17" s="7">
         <v>1018</v>
       </c>
-      <c r="L17" s="83">
+      <c r="M17" s="83">
         <v>16.064040000000002</v>
       </c>
-      <c r="M17" s="83">
+      <c r="N17" s="83">
         <v>0</v>
       </c>
-      <c r="N17" s="21">
+      <c r="O17" s="21">
         <v>35</v>
       </c>
-      <c r="O17" s="64">
+      <c r="P17" s="64">
         <v>8.76</v>
       </c>
-      <c r="P17" s="74">
+      <c r="Q17" s="74">
         <v>0.15309859852159369</v>
       </c>
-      <c r="R17" s="79"/>
-      <c r="T17" s="89" t="s">
+      <c r="S17" s="79"/>
+      <c r="U17" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V17" s="89" t="str">
+      <c r="W17" s="89" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$14,3)&amp;"_"&amp;Intra_areas!B7&amp;"00"</f>
         <v>ELCRESOL_JARVA00</v>
       </c>
-      <c r="W17" s="89" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V17,2)&amp;" in "&amp;Intra_areas!B7&amp;" - "&amp;'EB1'!$T$3</f>
+      <c r="X17" s="89" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W17,2)&amp;" in "&amp;Intra_areas!B7&amp;" - "&amp;'EB1'!$T$3</f>
         <v>Power Plants Existing00 in JARVA - Solar energy</v>
       </c>
-      <c r="X17" t="s">
+      <c r="Y17" t="s">
         <v>180</v>
       </c>
-      <c r="Y17" t="s">
+      <c r="Z17" t="s">
         <v>101</v>
       </c>
-      <c r="Z17" t="s">
+      <c r="AA17" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="18" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B18" s="21" t="str">
         <f t="shared" si="2"/>
         <v>ELCRESOL_JOGEVA00</v>
@@ -7759,53 +7866,56 @@
       <c r="G18">
         <v>4.7E-2</v>
       </c>
-      <c r="I18" s="93">
+      <c r="I18" s="7">
+        <v>2</v>
+      </c>
+      <c r="J18" s="93">
         <v>1</v>
       </c>
-      <c r="J18" s="63">
+      <c r="K18" s="63">
         <v>0.3</v>
       </c>
-      <c r="K18" s="7">
+      <c r="L18" s="7">
         <v>1018</v>
       </c>
-      <c r="L18" s="83">
+      <c r="M18" s="83">
         <v>16.064040000000002</v>
       </c>
-      <c r="M18" s="83">
+      <c r="N18" s="83">
         <v>0</v>
       </c>
-      <c r="N18" s="21">
+      <c r="O18" s="21">
         <v>35</v>
       </c>
-      <c r="O18" s="64">
+      <c r="P18" s="64">
         <v>8.76</v>
       </c>
-      <c r="P18" s="74">
+      <c r="Q18" s="74">
         <v>0.15309859852159369</v>
       </c>
-      <c r="R18" s="79"/>
-      <c r="T18" s="89" t="s">
+      <c r="S18" s="79"/>
+      <c r="U18" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V18" s="89" t="str">
+      <c r="W18" s="89" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$14,3)&amp;"_"&amp;Intra_areas!B8&amp;"00"</f>
         <v>ELCRESOL_JOGEVA00</v>
       </c>
-      <c r="W18" s="89" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V18,2)&amp;" in "&amp;Intra_areas!B8&amp;" - "&amp;'EB1'!$T$3</f>
+      <c r="X18" s="89" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W18,2)&amp;" in "&amp;Intra_areas!B8&amp;" - "&amp;'EB1'!$T$3</f>
         <v>Power Plants Existing00 in JOGEVA - Solar energy</v>
       </c>
-      <c r="X18" t="s">
+      <c r="Y18" t="s">
         <v>180</v>
       </c>
-      <c r="Y18" t="s">
+      <c r="Z18" t="s">
         <v>101</v>
       </c>
-      <c r="Z18" t="s">
+      <c r="AA18" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="19" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B19" s="21" t="str">
         <f t="shared" si="2"/>
         <v>ELCRESOL_HARJU00</v>
@@ -7821,52 +7931,55 @@
       <c r="G19">
         <v>0.04</v>
       </c>
-      <c r="I19" s="93">
+      <c r="I19" s="7">
+        <v>2</v>
+      </c>
+      <c r="J19" s="93">
         <v>1</v>
       </c>
-      <c r="J19" s="63">
+      <c r="K19" s="63">
         <v>0.3</v>
       </c>
-      <c r="K19" s="7">
+      <c r="L19" s="7">
         <v>1018</v>
       </c>
-      <c r="L19" s="83">
+      <c r="M19" s="83">
         <v>16.064040000000002</v>
       </c>
-      <c r="M19" s="83">
+      <c r="N19" s="83">
         <v>0</v>
       </c>
-      <c r="N19" s="21">
+      <c r="O19" s="21">
         <v>35</v>
       </c>
-      <c r="O19" s="64">
+      <c r="P19" s="64">
         <v>8.76</v>
       </c>
-      <c r="P19" s="74">
+      <c r="Q19" s="74">
         <v>0.15619560585976827</v>
       </c>
-      <c r="T19" s="89" t="s">
+      <c r="U19" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V19" s="89" t="str">
+      <c r="W19" s="89" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$14,3)&amp;"_"&amp;Intra_areas!B9&amp;"00"</f>
         <v>ELCRESOL_HARJU00</v>
       </c>
-      <c r="W19" s="89" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V19,2)&amp;" in "&amp;Intra_areas!B9&amp;" - "&amp;'EB1'!$T$3</f>
+      <c r="X19" s="89" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W19,2)&amp;" in "&amp;Intra_areas!B9&amp;" - "&amp;'EB1'!$T$3</f>
         <v>Power Plants Existing00 in HARJU - Solar energy</v>
       </c>
-      <c r="X19" t="s">
+      <c r="Y19" t="s">
         <v>180</v>
       </c>
-      <c r="Y19" t="s">
+      <c r="Z19" t="s">
         <v>101</v>
       </c>
-      <c r="Z19" t="s">
+      <c r="AA19" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="20" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B20" s="21" t="str">
         <f t="shared" si="2"/>
         <v>ELCRESOL_POLVA00</v>
@@ -7882,52 +7995,55 @@
       <c r="G20">
         <v>0.24199999999999999</v>
       </c>
-      <c r="I20" s="93">
+      <c r="I20" s="7">
+        <v>2</v>
+      </c>
+      <c r="J20" s="93">
         <v>1</v>
       </c>
-      <c r="J20" s="63">
+      <c r="K20" s="63">
         <v>0.3</v>
       </c>
-      <c r="K20" s="7">
+      <c r="L20" s="7">
         <v>1018</v>
       </c>
-      <c r="L20" s="83">
+      <c r="M20" s="83">
         <v>16.064040000000002</v>
       </c>
-      <c r="M20" s="83">
+      <c r="N20" s="83">
         <v>0</v>
       </c>
-      <c r="N20" s="21">
+      <c r="O20" s="21">
         <v>35</v>
       </c>
-      <c r="O20" s="64">
+      <c r="P20" s="64">
         <v>8.76</v>
       </c>
-      <c r="P20" s="74">
+      <c r="Q20" s="74">
         <v>0.14537310453496291</v>
       </c>
-      <c r="T20" s="89" t="s">
+      <c r="U20" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V20" s="89" t="str">
+      <c r="W20" s="89" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$14,3)&amp;"_"&amp;Intra_areas!B10&amp;"00"</f>
         <v>ELCRESOL_POLVA00</v>
       </c>
-      <c r="W20" s="89" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V20,2)&amp;" in "&amp;Intra_areas!B10&amp;" - "&amp;'EB1'!$T$3</f>
+      <c r="X20" s="89" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W20,2)&amp;" in "&amp;Intra_areas!B10&amp;" - "&amp;'EB1'!$T$3</f>
         <v>Power Plants Existing00 in POLVA - Solar energy</v>
       </c>
-      <c r="X20" t="s">
+      <c r="Y20" t="s">
         <v>180</v>
       </c>
-      <c r="Y20" t="s">
+      <c r="Z20" t="s">
         <v>101</v>
       </c>
-      <c r="Z20" t="s">
+      <c r="AA20" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="21" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B21" s="21" t="str">
         <f t="shared" si="2"/>
         <v>ELCRESOL_VALGA00</v>
@@ -7943,52 +8059,55 @@
       <c r="G21">
         <v>4.2999999999999997E-2</v>
       </c>
-      <c r="I21" s="93">
+      <c r="I21" s="7">
+        <v>2</v>
+      </c>
+      <c r="J21" s="93">
         <v>1</v>
       </c>
-      <c r="J21" s="63">
+      <c r="K21" s="63">
         <v>0.3</v>
       </c>
-      <c r="K21" s="7">
+      <c r="L21" s="7">
         <v>1018</v>
       </c>
-      <c r="L21" s="83">
+      <c r="M21" s="83">
         <v>16.064040000000002</v>
       </c>
-      <c r="M21" s="83">
+      <c r="N21" s="83">
         <v>0</v>
       </c>
-      <c r="N21" s="21">
+      <c r="O21" s="21">
         <v>35</v>
       </c>
-      <c r="O21" s="64">
+      <c r="P21" s="64">
         <v>8.76</v>
       </c>
-      <c r="P21" s="74">
+      <c r="Q21" s="74">
         <v>0.14763873655681015</v>
       </c>
-      <c r="T21" s="89" t="s">
+      <c r="U21" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V21" s="89" t="str">
+      <c r="W21" s="89" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$14,3)&amp;"_"&amp;Intra_areas!B11&amp;"00"</f>
         <v>ELCRESOL_VALGA00</v>
       </c>
-      <c r="W21" s="89" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V21,2)&amp;" in "&amp;Intra_areas!B11&amp;" - "&amp;'EB1'!$T$3</f>
+      <c r="X21" s="89" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W21,2)&amp;" in "&amp;Intra_areas!B11&amp;" - "&amp;'EB1'!$T$3</f>
         <v>Power Plants Existing00 in VALGA - Solar energy</v>
       </c>
-      <c r="X21" t="s">
+      <c r="Y21" t="s">
         <v>180</v>
       </c>
-      <c r="Y21" t="s">
+      <c r="Z21" t="s">
         <v>101</v>
       </c>
-      <c r="Z21" t="s">
+      <c r="AA21" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="22" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B22" s="21" t="str">
         <f t="shared" si="2"/>
         <v>ELCRESOL_VILJANDI00</v>
@@ -8004,52 +8123,55 @@
       <c r="G22">
         <v>0.08</v>
       </c>
-      <c r="I22" s="93">
+      <c r="I22" s="7">
+        <v>2</v>
+      </c>
+      <c r="J22" s="93">
         <v>1</v>
       </c>
-      <c r="J22" s="63">
+      <c r="K22" s="63">
         <v>0.3</v>
       </c>
-      <c r="K22" s="7">
+      <c r="L22" s="7">
         <v>1018</v>
       </c>
-      <c r="L22" s="83">
+      <c r="M22" s="83">
         <v>16.064040000000002</v>
       </c>
-      <c r="M22" s="83">
+      <c r="N22" s="83">
         <v>0</v>
       </c>
-      <c r="N22" s="21">
+      <c r="O22" s="21">
         <v>35</v>
       </c>
-      <c r="O22" s="64">
+      <c r="P22" s="64">
         <v>8.76</v>
       </c>
-      <c r="P22" s="74">
+      <c r="Q22" s="74">
         <v>0.1532628310027955</v>
       </c>
-      <c r="T22" s="89" t="s">
+      <c r="U22" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V22" s="89" t="str">
+      <c r="W22" s="89" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$14,3)&amp;"_"&amp;Intra_areas!B12&amp;"00"</f>
         <v>ELCRESOL_VILJANDI00</v>
       </c>
-      <c r="W22" s="89" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V22,2)&amp;" in "&amp;Intra_areas!B12&amp;" - "&amp;'EB1'!$T$3</f>
+      <c r="X22" s="89" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W22,2)&amp;" in "&amp;Intra_areas!B12&amp;" - "&amp;'EB1'!$T$3</f>
         <v>Power Plants Existing00 in VILJANDI - Solar energy</v>
       </c>
-      <c r="X22" t="s">
+      <c r="Y22" t="s">
         <v>180</v>
       </c>
-      <c r="Y22" t="s">
+      <c r="Z22" t="s">
         <v>101</v>
       </c>
-      <c r="Z22" t="s">
+      <c r="AA22" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="23" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B23" s="21" t="str">
         <f t="shared" si="2"/>
         <v>ELCRESOL_VORU00</v>
@@ -8065,52 +8187,55 @@
       <c r="G23">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="I23" s="93">
+      <c r="I23" s="7">
+        <v>2</v>
+      </c>
+      <c r="J23" s="93">
         <v>1</v>
       </c>
-      <c r="J23" s="63">
+      <c r="K23" s="63">
         <v>0.3</v>
       </c>
-      <c r="K23" s="7">
+      <c r="L23" s="7">
         <v>1019</v>
       </c>
-      <c r="L23" s="83">
+      <c r="M23" s="83">
         <v>16.079820000000002</v>
       </c>
-      <c r="M23" s="83">
+      <c r="N23" s="83">
         <v>0</v>
       </c>
-      <c r="N23" s="21">
+      <c r="O23" s="21">
         <v>35</v>
       </c>
-      <c r="O23" s="64">
+      <c r="P23" s="64">
         <v>8.76</v>
       </c>
-      <c r="P23" s="74">
+      <c r="Q23" s="74">
         <v>0.1461854238754417</v>
       </c>
-      <c r="T23" s="89" t="s">
+      <c r="U23" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V23" s="89" t="str">
+      <c r="W23" s="89" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$14,3)&amp;"_"&amp;Intra_areas!B13&amp;"00"</f>
         <v>ELCRESOL_VORU00</v>
       </c>
-      <c r="W23" s="89" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V23,2)&amp;" in "&amp;Intra_areas!B13&amp;" - "&amp;'EB1'!$T$3</f>
+      <c r="X23" s="89" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W23,2)&amp;" in "&amp;Intra_areas!B13&amp;" - "&amp;'EB1'!$T$3</f>
         <v>Power Plants Existing00 in VORU - Solar energy</v>
       </c>
-      <c r="X23" t="s">
+      <c r="Y23" t="s">
         <v>180</v>
       </c>
-      <c r="Y23" t="s">
+      <c r="Z23" t="s">
         <v>101</v>
       </c>
-      <c r="Z23" t="s">
+      <c r="AA23" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="24" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B24" s="21" t="str">
         <f t="shared" si="2"/>
         <v>ELCRESOL_SAARE00</v>
@@ -8126,52 +8251,55 @@
       <c r="G24">
         <v>3.1E-2</v>
       </c>
-      <c r="I24" s="93">
+      <c r="I24" s="7">
+        <v>2</v>
+      </c>
+      <c r="J24" s="93">
         <v>1</v>
       </c>
-      <c r="J24" s="63">
+      <c r="K24" s="63">
         <v>0.3</v>
       </c>
-      <c r="K24" s="7">
+      <c r="L24" s="7">
         <v>1020</v>
       </c>
-      <c r="L24" s="83">
+      <c r="M24" s="83">
         <v>16.095600000000001</v>
       </c>
-      <c r="M24" s="83">
+      <c r="N24" s="83">
         <v>0</v>
       </c>
-      <c r="N24" s="21">
+      <c r="O24" s="21">
         <v>35</v>
       </c>
-      <c r="O24" s="64">
+      <c r="P24" s="64">
         <v>8.76</v>
       </c>
-      <c r="P24" s="74">
+      <c r="Q24" s="74">
         <v>0.1461854238754417</v>
       </c>
-      <c r="T24" s="89" t="s">
+      <c r="U24" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V24" s="89" t="str">
+      <c r="W24" s="89" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$14,3)&amp;"_"&amp;Intra_areas!B14&amp;"00"</f>
         <v>ELCRESOL_SAARE00</v>
       </c>
-      <c r="W24" s="89" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V24,2)&amp;" in "&amp;Intra_areas!B14&amp;" - "&amp;'EB1'!$T$3</f>
+      <c r="X24" s="89" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W24,2)&amp;" in "&amp;Intra_areas!B14&amp;" - "&amp;'EB1'!$T$3</f>
         <v>Power Plants Existing00 in SAARE - Solar energy</v>
       </c>
-      <c r="X24" t="s">
+      <c r="Y24" t="s">
         <v>180</v>
       </c>
-      <c r="Y24" t="s">
+      <c r="Z24" t="s">
         <v>101</v>
       </c>
-      <c r="Z24" t="s">
+      <c r="AA24" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="25" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B25" s="21" t="str">
         <f t="shared" si="2"/>
         <v>ELCRESOL_RAPLA00</v>
@@ -8187,52 +8315,55 @@
       <c r="G25">
         <v>2.9000000000000001E-2</v>
       </c>
-      <c r="I25" s="93">
+      <c r="I25" s="7">
+        <v>2</v>
+      </c>
+      <c r="J25" s="93">
         <v>1</v>
       </c>
-      <c r="J25" s="63">
+      <c r="K25" s="63">
         <v>0.3</v>
       </c>
-      <c r="K25" s="7">
+      <c r="L25" s="7">
         <v>1021</v>
       </c>
-      <c r="L25" s="83">
+      <c r="M25" s="83">
         <v>16.111380000000004</v>
       </c>
-      <c r="M25" s="83">
+      <c r="N25" s="83">
         <v>0</v>
       </c>
-      <c r="N25" s="21">
+      <c r="O25" s="21">
         <v>35</v>
       </c>
-      <c r="O25" s="64">
+      <c r="P25" s="64">
         <v>8.76</v>
       </c>
-      <c r="P25" s="74">
+      <c r="Q25" s="74">
         <v>0.1461854238754417</v>
       </c>
-      <c r="T25" s="89" t="s">
+      <c r="U25" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V25" s="89" t="str">
+      <c r="W25" s="89" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$14,3)&amp;"_"&amp;Intra_areas!B15&amp;"00"</f>
         <v>ELCRESOL_RAPLA00</v>
       </c>
-      <c r="W25" s="89" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V25,2)&amp;" in "&amp;Intra_areas!B15&amp;" - "&amp;'EB1'!$T$3</f>
+      <c r="X25" s="89" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W25,2)&amp;" in "&amp;Intra_areas!B15&amp;" - "&amp;'EB1'!$T$3</f>
         <v>Power Plants Existing00 in RAPLA - Solar energy</v>
       </c>
-      <c r="X25" t="s">
+      <c r="Y25" t="s">
         <v>180</v>
       </c>
-      <c r="Y25" t="s">
+      <c r="Z25" t="s">
         <v>101</v>
       </c>
-      <c r="Z25" t="s">
+      <c r="AA25" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="26" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B26" s="21" t="str">
         <f t="shared" si="2"/>
         <v>ELCRESOL_LAANE00</v>
@@ -8248,52 +8379,55 @@
       <c r="G26">
         <v>0.01</v>
       </c>
-      <c r="I26" s="93">
+      <c r="I26" s="7">
+        <v>2</v>
+      </c>
+      <c r="J26" s="93">
         <v>1</v>
       </c>
-      <c r="J26" s="63">
+      <c r="K26" s="63">
         <v>0.3</v>
       </c>
-      <c r="K26" s="7">
+      <c r="L26" s="7">
         <v>1022</v>
       </c>
-      <c r="L26" s="83">
+      <c r="M26" s="83">
         <v>16.127160000000003</v>
       </c>
-      <c r="M26" s="83">
+      <c r="N26" s="83">
         <v>0</v>
       </c>
-      <c r="N26" s="21">
+      <c r="O26" s="21">
         <v>35</v>
       </c>
-      <c r="O26" s="64">
+      <c r="P26" s="64">
         <v>8.76</v>
       </c>
-      <c r="P26" s="74">
+      <c r="Q26" s="74">
         <v>0.1461854238754417</v>
       </c>
-      <c r="T26" s="89" t="s">
+      <c r="U26" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V26" s="89" t="str">
+      <c r="W26" s="89" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$14,3)&amp;"_"&amp;Intra_areas!B16&amp;"00"</f>
         <v>ELCRESOL_LAANE00</v>
       </c>
-      <c r="W26" s="89" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V26,2)&amp;" in "&amp;Intra_areas!B16&amp;" - "&amp;'EB1'!$T$3</f>
+      <c r="X26" s="89" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W26,2)&amp;" in "&amp;Intra_areas!B16&amp;" - "&amp;'EB1'!$T$3</f>
         <v>Power Plants Existing00 in LAANE - Solar energy</v>
       </c>
-      <c r="X26" t="s">
+      <c r="Y26" t="s">
         <v>180</v>
       </c>
-      <c r="Y26" t="s">
+      <c r="Z26" t="s">
         <v>101</v>
       </c>
-      <c r="Z26" t="s">
+      <c r="AA26" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="27" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B27" s="21" t="str">
         <f t="shared" si="2"/>
         <v>ELCRESOL_HIIU00</v>
@@ -8309,52 +8443,55 @@
       <c r="G27">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="I27" s="93">
+      <c r="I27" s="7">
+        <v>2</v>
+      </c>
+      <c r="J27" s="93">
         <v>1</v>
       </c>
-      <c r="J27" s="63">
+      <c r="K27" s="63">
         <v>0.3</v>
       </c>
-      <c r="K27" s="7">
+      <c r="L27" s="7">
         <v>1023</v>
       </c>
-      <c r="L27" s="83">
+      <c r="M27" s="83">
         <v>16.142940000000003</v>
       </c>
-      <c r="M27" s="83">
+      <c r="N27" s="83">
         <v>0</v>
       </c>
-      <c r="N27" s="21">
+      <c r="O27" s="21">
         <v>35</v>
       </c>
-      <c r="O27" s="21">
+      <c r="P27" s="21">
         <v>8.76</v>
       </c>
-      <c r="P27" s="74">
+      <c r="Q27" s="74">
         <v>0.1461854238754417</v>
       </c>
-      <c r="T27" s="89" t="s">
+      <c r="U27" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V27" s="89" t="str">
+      <c r="W27" s="89" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$14,3)&amp;"_"&amp;Intra_areas!B17&amp;"00"</f>
         <v>ELCRESOL_HIIU00</v>
       </c>
-      <c r="W27" s="89" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V27,2)&amp;" in "&amp;Intra_areas!B17&amp;" - "&amp;'EB1'!$T$3</f>
+      <c r="X27" s="89" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W27,2)&amp;" in "&amp;Intra_areas!B17&amp;" - "&amp;'EB1'!$T$3</f>
         <v>Power Plants Existing00 in HIIU - Solar energy</v>
       </c>
-      <c r="X27" t="s">
+      <c r="Y27" t="s">
         <v>180</v>
       </c>
-      <c r="Y27" t="s">
+      <c r="Z27" t="s">
         <v>101</v>
       </c>
-      <c r="Z27" t="s">
+      <c r="AA27" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="28" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B28" s="21" t="str">
         <f t="shared" si="2"/>
         <v>ELCREWON_SOPITOOTSI00</v>
@@ -8370,52 +8507,55 @@
       <c r="G28">
         <v>7.9699999999999993E-2</v>
       </c>
-      <c r="I28" s="93">
+      <c r="I28" s="7">
+        <v>2</v>
+      </c>
+      <c r="J28" s="93">
         <v>1</v>
       </c>
-      <c r="J28" s="63">
+      <c r="K28" s="63">
         <v>0.3</v>
       </c>
-      <c r="K28" s="7">
+      <c r="L28" s="7">
         <v>1494.4630999999999</v>
       </c>
-      <c r="L28" s="83">
+      <c r="M28" s="83">
         <v>18.701711233400001</v>
       </c>
-      <c r="M28" s="83">
+      <c r="N28" s="83">
         <v>2.0036999999999998</v>
       </c>
-      <c r="N28">
+      <c r="O28">
         <v>27</v>
       </c>
-      <c r="O28" s="21">
+      <c r="P28" s="21">
         <v>8.76</v>
       </c>
-      <c r="P28">
+      <c r="Q28">
         <v>0.4</v>
       </c>
-      <c r="T28" s="89" t="s">
+      <c r="U28" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V28" t="str">
+      <c r="W28" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)&amp;"_"&amp;Intra_areas!C3&amp;"00"</f>
         <v>ELCREWON_SOPITOOTSI00</v>
       </c>
-      <c r="W28" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V28,2)&amp;" in "&amp;Intra_areas!C3&amp;" - "&amp;'EB1'!$R$3</f>
+      <c r="X28" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W28,2)&amp;" in "&amp;Intra_areas!C3&amp;" - "&amp;'EB1'!$R$3</f>
         <v>Power Plants Existing00 in SOPITOOTSI - Wind onshore energy</v>
       </c>
-      <c r="X28" t="s">
+      <c r="Y28" t="s">
         <v>180</v>
       </c>
-      <c r="Y28" t="s">
+      <c r="Z28" t="s">
         <v>101</v>
       </c>
-      <c r="Z28" t="s">
+      <c r="AA28" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="29" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B29" s="21" t="str">
         <f t="shared" si="2"/>
         <v>ELCREWON_SOPIPURTSE00</v>
@@ -8431,52 +8571,55 @@
       <c r="G29">
         <v>0.17519999999999999</v>
       </c>
-      <c r="I29" s="93">
+      <c r="I29" s="7">
+        <v>2</v>
+      </c>
+      <c r="J29" s="93">
         <v>1</v>
       </c>
-      <c r="J29" s="63">
+      <c r="K29" s="63">
         <v>0.3</v>
       </c>
-      <c r="K29" s="7">
+      <c r="L29" s="7">
         <v>1494.4630999999999</v>
       </c>
-      <c r="L29" s="83">
+      <c r="M29" s="83">
         <v>18.701711233400001</v>
       </c>
-      <c r="M29" s="83">
+      <c r="N29" s="83">
         <v>2.0036999999999998</v>
       </c>
-      <c r="N29">
+      <c r="O29">
         <v>27</v>
       </c>
-      <c r="O29" s="21">
+      <c r="P29" s="21">
         <v>8.76</v>
       </c>
-      <c r="P29">
+      <c r="Q29">
         <v>0.4</v>
       </c>
-      <c r="T29" s="89" t="s">
+      <c r="U29" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V29" t="str">
+      <c r="W29" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)&amp;"_"&amp;Intra_areas!C4&amp;"00"</f>
         <v>ELCREWON_SOPIPURTSE00</v>
       </c>
-      <c r="W29" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V29,2)&amp;" in "&amp;Intra_areas!C4&amp;" - "&amp;'EB1'!$R$3</f>
+      <c r="X29" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W29,2)&amp;" in "&amp;Intra_areas!C4&amp;" - "&amp;'EB1'!$R$3</f>
         <v>Power Plants Existing00 in SOPIPURTSE - Wind onshore energy</v>
       </c>
-      <c r="X29" t="s">
+      <c r="Y29" t="s">
         <v>180</v>
       </c>
-      <c r="Y29" t="s">
+      <c r="Z29" t="s">
         <v>101</v>
       </c>
-      <c r="Z29" t="s">
+      <c r="AA29" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="30" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B30" s="21" t="str">
         <f t="shared" si="2"/>
         <v>ELCREWON_OTHER00</v>
@@ -8492,52 +8635,55 @@
       <c r="G30">
         <v>8.130000000000015E-2</v>
       </c>
-      <c r="I30" s="93">
+      <c r="I30" s="7">
+        <v>2</v>
+      </c>
+      <c r="J30" s="93">
         <v>1</v>
       </c>
-      <c r="J30" s="63">
+      <c r="K30" s="63">
         <v>0.3</v>
       </c>
-      <c r="K30" s="7">
+      <c r="L30" s="7">
         <v>1494.4630999999999</v>
       </c>
-      <c r="L30" s="83">
+      <c r="M30" s="83">
         <v>18.701711233400001</v>
       </c>
-      <c r="M30" s="83">
+      <c r="N30" s="83">
         <v>2.0036999999999998</v>
       </c>
-      <c r="N30">
+      <c r="O30">
         <v>27</v>
       </c>
-      <c r="O30" s="21">
+      <c r="P30" s="21">
         <v>8.76</v>
       </c>
-      <c r="P30">
+      <c r="Q30">
         <v>0.4</v>
       </c>
-      <c r="T30" s="89" t="s">
+      <c r="U30" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V30" t="str">
+      <c r="W30" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)&amp;"_"&amp;Intra_areas!C5&amp;"00"</f>
         <v>ELCREWON_OTHER00</v>
       </c>
-      <c r="W30" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V30,2)&amp;" in "&amp;Intra_areas!C5&amp;" - "&amp;'EB1'!$R$3</f>
+      <c r="X30" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W30,2)&amp;" in "&amp;Intra_areas!C5&amp;" - "&amp;'EB1'!$R$3</f>
         <v>Power Plants Existing00 in OTHER - Wind onshore energy</v>
       </c>
-      <c r="X30" t="s">
+      <c r="Y30" t="s">
         <v>180</v>
       </c>
-      <c r="Y30" t="s">
+      <c r="Z30" t="s">
         <v>101</v>
       </c>
-      <c r="Z30" t="s">
+      <c r="AA30" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="31" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B31" s="21" t="str">
         <f t="shared" si="2"/>
         <v>ELCREWON_SAARE00</v>
@@ -8553,52 +8699,55 @@
       <c r="G31">
         <v>1.6E-2</v>
       </c>
-      <c r="I31" s="93">
+      <c r="I31" s="7">
+        <v>2</v>
+      </c>
+      <c r="J31" s="93">
         <v>1</v>
       </c>
-      <c r="J31" s="63">
+      <c r="K31" s="63">
         <v>0.3</v>
       </c>
-      <c r="K31" s="7">
+      <c r="L31" s="7">
         <v>1494.4630999999999</v>
       </c>
-      <c r="L31" s="83">
+      <c r="M31" s="83">
         <v>18.701711233400001</v>
       </c>
-      <c r="M31" s="83">
+      <c r="N31" s="83">
         <v>2.0036999999999998</v>
       </c>
-      <c r="N31">
+      <c r="O31">
         <v>27</v>
       </c>
-      <c r="O31" s="21">
+      <c r="P31" s="21">
         <v>8.76</v>
       </c>
-      <c r="P31">
+      <c r="Q31">
         <v>0.4</v>
       </c>
-      <c r="T31" s="89" t="s">
+      <c r="U31" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V31" t="str">
+      <c r="W31" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)&amp;"_"&amp;Intra_areas!C6&amp;"00"</f>
         <v>ELCREWON_SAARE00</v>
       </c>
-      <c r="W31" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V31,2)&amp;" in "&amp;Intra_areas!C6&amp;" - "&amp;'EB1'!$R$3</f>
+      <c r="X31" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W31,2)&amp;" in "&amp;Intra_areas!C6&amp;" - "&amp;'EB1'!$R$3</f>
         <v>Power Plants Existing00 in SAARE - Wind onshore energy</v>
       </c>
-      <c r="X31" t="s">
+      <c r="Y31" t="s">
         <v>180</v>
       </c>
-      <c r="Y31" t="s">
+      <c r="Z31" t="s">
         <v>101</v>
       </c>
-      <c r="Z31" t="s">
+      <c r="AA31" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="32" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B32" s="21" t="str">
         <f t="shared" si="2"/>
         <v>ELCREWON_LVIRU00</v>
@@ -8614,52 +8763,55 @@
       <c r="G32">
         <v>3.27E-2</v>
       </c>
-      <c r="I32" s="93">
+      <c r="I32" s="7">
+        <v>2</v>
+      </c>
+      <c r="J32" s="93">
         <v>1</v>
       </c>
-      <c r="J32" s="63">
+      <c r="K32" s="63">
         <v>0.3</v>
       </c>
-      <c r="K32" s="7">
+      <c r="L32" s="7">
         <v>1494.4630999999999</v>
       </c>
-      <c r="L32" s="83">
+      <c r="M32" s="83">
         <v>18.701711233400001</v>
       </c>
-      <c r="M32" s="83">
+      <c r="N32" s="83">
         <v>2.0036999999999998</v>
       </c>
-      <c r="N32">
+      <c r="O32">
         <v>27</v>
       </c>
-      <c r="O32" s="21">
+      <c r="P32" s="21">
         <v>8.76</v>
       </c>
-      <c r="P32">
+      <c r="Q32">
         <v>0.4</v>
       </c>
-      <c r="T32" s="89" t="s">
+      <c r="U32" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V32" t="str">
+      <c r="W32" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)&amp;"_"&amp;Intra_areas!C7&amp;"00"</f>
         <v>ELCREWON_LVIRU00</v>
       </c>
-      <c r="W32" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V32,2)&amp;" in "&amp;Intra_areas!C7&amp;" - "&amp;'EB1'!$R$3</f>
+      <c r="X32" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W32,2)&amp;" in "&amp;Intra_areas!C7&amp;" - "&amp;'EB1'!$R$3</f>
         <v>Power Plants Existing00 in LVIRU - Wind onshore energy</v>
       </c>
-      <c r="X32" t="s">
+      <c r="Y32" t="s">
         <v>180</v>
       </c>
-      <c r="Y32" t="s">
+      <c r="Z32" t="s">
         <v>101</v>
       </c>
-      <c r="Z32" t="s">
+      <c r="AA32" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="33" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B33" s="21" t="str">
         <f t="shared" si="2"/>
         <v>ELCREWON_HARJU00</v>
@@ -8675,52 +8827,55 @@
       <c r="G33">
         <v>6.3399999999999998E-2</v>
       </c>
-      <c r="I33" s="93">
+      <c r="I33" s="7">
+        <v>2</v>
+      </c>
+      <c r="J33" s="93">
         <v>1</v>
       </c>
-      <c r="J33" s="63">
+      <c r="K33" s="63">
         <v>0.3</v>
       </c>
-      <c r="K33" s="7">
+      <c r="L33" s="7">
         <v>1494.4630999999999</v>
       </c>
-      <c r="L33" s="83">
+      <c r="M33" s="83">
         <v>18.701711233400001</v>
       </c>
-      <c r="M33" s="83">
+      <c r="N33" s="83">
         <v>2.0036999999999998</v>
       </c>
-      <c r="N33">
+      <c r="O33">
         <v>27</v>
       </c>
-      <c r="O33" s="21">
+      <c r="P33" s="21">
         <v>8.76</v>
       </c>
-      <c r="P33">
+      <c r="Q33">
         <v>0.4</v>
       </c>
-      <c r="T33" s="89" t="s">
+      <c r="U33" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V33" t="str">
+      <c r="W33" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)&amp;"_"&amp;Intra_areas!C8&amp;"00"</f>
         <v>ELCREWON_HARJU00</v>
       </c>
-      <c r="W33" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V33,2)&amp;" in "&amp;Intra_areas!C8&amp;" - "&amp;'EB1'!$R$3</f>
+      <c r="X33" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W33,2)&amp;" in "&amp;Intra_areas!C8&amp;" - "&amp;'EB1'!$R$3</f>
         <v>Power Plants Existing00 in HARJU - Wind onshore energy</v>
       </c>
-      <c r="X33" t="s">
+      <c r="Y33" t="s">
         <v>180</v>
       </c>
-      <c r="Y33" t="s">
+      <c r="Z33" t="s">
         <v>101</v>
       </c>
-      <c r="Z33" t="s">
+      <c r="AA33" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="34" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B34" s="21" t="str">
         <f t="shared" si="2"/>
         <v>ELCREWON_LAANE00</v>
@@ -8736,52 +8891,55 @@
       <c r="G34">
         <v>0.06</v>
       </c>
-      <c r="I34" s="93">
+      <c r="I34" s="7">
+        <v>2</v>
+      </c>
+      <c r="J34" s="93">
         <v>1</v>
       </c>
-      <c r="J34" s="63">
+      <c r="K34" s="63">
         <v>0.3</v>
       </c>
-      <c r="K34" s="7">
+      <c r="L34" s="7">
         <v>1494.4630999999999</v>
       </c>
-      <c r="L34" s="83">
+      <c r="M34" s="83">
         <v>18.701711233400001</v>
       </c>
-      <c r="M34" s="83">
+      <c r="N34" s="83">
         <v>2.0036999999999998</v>
       </c>
-      <c r="N34">
+      <c r="O34">
         <v>27</v>
       </c>
-      <c r="O34" s="21">
+      <c r="P34" s="21">
         <v>8.76</v>
       </c>
-      <c r="P34">
+      <c r="Q34">
         <v>0.4</v>
       </c>
-      <c r="T34" s="89" t="s">
+      <c r="U34" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V34" t="str">
+      <c r="W34" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)&amp;"_"&amp;Intra_areas!C9&amp;"00"</f>
         <v>ELCREWON_LAANE00</v>
       </c>
-      <c r="W34" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V34,2)&amp;" in "&amp;Intra_areas!C9&amp;" - "&amp;'EB1'!$R$3</f>
+      <c r="X34" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W34,2)&amp;" in "&amp;Intra_areas!C9&amp;" - "&amp;'EB1'!$R$3</f>
         <v>Power Plants Existing00 in LAANE - Wind onshore energy</v>
       </c>
-      <c r="X34" t="s">
+      <c r="Y34" t="s">
         <v>180</v>
       </c>
-      <c r="Y34" t="s">
+      <c r="Z34" t="s">
         <v>101</v>
       </c>
-      <c r="Z34" t="s">
+      <c r="AA34" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="35" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B35" s="21" t="str">
         <f t="shared" si="2"/>
         <v>ELCREWON_IVIRU00</v>
@@ -8797,52 +8955,55 @@
       <c r="G35">
         <v>8.2000000000000003E-2</v>
       </c>
-      <c r="I35" s="93">
+      <c r="I35" s="7">
+        <v>2</v>
+      </c>
+      <c r="J35" s="93">
         <v>1</v>
       </c>
-      <c r="J35" s="63">
+      <c r="K35" s="63">
         <v>0.3</v>
       </c>
-      <c r="K35" s="7">
+      <c r="L35" s="7">
         <v>1494.4630999999999</v>
       </c>
-      <c r="L35" s="83">
+      <c r="M35" s="83">
         <v>18.701711233400001</v>
       </c>
-      <c r="M35" s="83">
+      <c r="N35" s="83">
         <v>2.0036999999999998</v>
       </c>
-      <c r="N35">
+      <c r="O35">
         <v>27</v>
       </c>
-      <c r="O35" s="21">
+      <c r="P35" s="21">
         <v>8.76</v>
       </c>
-      <c r="P35">
+      <c r="Q35">
         <v>0.4</v>
       </c>
-      <c r="T35" s="89" t="s">
+      <c r="U35" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V35" t="str">
+      <c r="W35" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)&amp;"_"&amp;Intra_areas!C10&amp;"00"</f>
         <v>ELCREWON_IVIRU00</v>
       </c>
-      <c r="W35" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V35,2)&amp;" in "&amp;Intra_areas!C10&amp;" - "&amp;'EB1'!$R$3</f>
+      <c r="X35" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W35,2)&amp;" in "&amp;Intra_areas!C10&amp;" - "&amp;'EB1'!$R$3</f>
         <v>Power Plants Existing00 in IVIRU - Wind onshore energy</v>
       </c>
-      <c r="X35" t="s">
+      <c r="Y35" t="s">
         <v>180</v>
       </c>
-      <c r="Y35" t="s">
+      <c r="Z35" t="s">
         <v>101</v>
       </c>
-      <c r="Z35" t="s">
+      <c r="AA35" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="36" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B36" s="21" t="str">
         <f t="shared" si="2"/>
         <v>ELCREWON_PARNU00</v>
@@ -8858,52 +9019,55 @@
       <c r="G36">
         <v>0.1036</v>
       </c>
-      <c r="I36" s="93">
+      <c r="I36" s="7">
+        <v>2</v>
+      </c>
+      <c r="J36" s="93">
         <v>1</v>
       </c>
-      <c r="J36" s="63">
+      <c r="K36" s="63">
         <v>0.3</v>
       </c>
-      <c r="K36" s="7">
+      <c r="L36" s="7">
         <v>1494.4630999999999</v>
       </c>
-      <c r="L36" s="83">
+      <c r="M36" s="83">
         <v>18.701711233400001</v>
       </c>
-      <c r="M36" s="83">
+      <c r="N36" s="83">
         <v>2.0036999999999998</v>
       </c>
-      <c r="N36">
+      <c r="O36">
         <v>27</v>
       </c>
-      <c r="O36" s="21">
+      <c r="P36" s="21">
         <v>8.76</v>
       </c>
-      <c r="P36">
+      <c r="Q36">
         <v>0.4</v>
       </c>
-      <c r="T36" s="89" t="s">
+      <c r="U36" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V36" t="str">
+      <c r="W36" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$12,3)&amp;"_"&amp;Intra_areas!C11&amp;"00"</f>
         <v>ELCREWON_PARNU00</v>
       </c>
-      <c r="W36" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V36,2)&amp;" in "&amp;Intra_areas!C11&amp;" - "&amp;'EB1'!$R$3</f>
+      <c r="X36" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W36,2)&amp;" in "&amp;Intra_areas!C11&amp;" - "&amp;'EB1'!$R$3</f>
         <v>Power Plants Existing00 in PARNU - Wind onshore energy</v>
       </c>
-      <c r="X36" t="s">
+      <c r="Y36" t="s">
         <v>180</v>
       </c>
-      <c r="Y36" t="s">
+      <c r="Z36" t="s">
         <v>101</v>
       </c>
-      <c r="Z36" t="s">
+      <c r="AA36" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="37" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="37" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B37" s="21" t="str">
         <f t="shared" si="2"/>
         <v>ELCREMSW_IRU00</v>
@@ -8919,54 +9083,57 @@
       <c r="G37" s="21">
         <v>1.7000000000000001E-2</v>
       </c>
-      <c r="I37" s="21">
+      <c r="I37" s="7">
+        <v>2</v>
+      </c>
+      <c r="J37" s="21">
         <v>0.56000000000000005</v>
       </c>
-      <c r="J37" s="21">
+      <c r="K37" s="21">
         <v>0.9</v>
       </c>
-      <c r="K37" s="79">
+      <c r="L37" s="79">
         <v>1175.5066999999999</v>
       </c>
-      <c r="L37" s="79">
+      <c r="M37" s="79">
         <v>160.216352398</v>
       </c>
-      <c r="M37" s="79">
+      <c r="N37" s="79">
         <v>5.8775000000000004</v>
       </c>
-      <c r="N37" s="79">
+      <c r="O37" s="79">
         <v>53</v>
       </c>
-      <c r="O37" s="21">
+      <c r="P37" s="21">
         <v>8.76</v>
       </c>
-      <c r="P37">
+      <c r="Q37">
         <v>1</v>
       </c>
-      <c r="T37" s="89" t="s">
+      <c r="U37" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V37" t="str">
+      <c r="W37" t="str">
         <f>$B$2&amp;$E$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!L15,3)&amp;"_IRU"&amp;"00"</f>
         <v>ELCREMSW_IRU00</v>
       </c>
-      <c r="W37" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V37,2)&amp;" Iru Power plant - Municipal waste"</f>
+      <c r="X37" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W37,2)&amp;" Iru Power plant - Municipal waste"</f>
         <v>Power Plants Existing00 Iru Power plant - Municipal waste</v>
       </c>
-      <c r="X37" t="s">
+      <c r="Y37" t="s">
         <v>180</v>
       </c>
-      <c r="Y37" t="s">
+      <c r="Z37" t="s">
         <v>101</v>
       </c>
-      <c r="Z37" t="s">
+      <c r="AA37" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="38" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="38" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B38" s="21" t="str">
-        <f>V38</f>
+        <f>W38</f>
         <v>ELCTESHL_EESTI00</v>
       </c>
       <c r="C38" s="21" t="str">
@@ -8980,55 +9147,58 @@
       <c r="G38" s="21">
         <v>0.77</v>
       </c>
-      <c r="I38" s="21">
+      <c r="I38" s="7">
+        <v>2</v>
+      </c>
+      <c r="J38" s="21">
         <v>0.33</v>
       </c>
-      <c r="J38" s="21">
+      <c r="K38" s="21">
         <v>0.95</v>
       </c>
-      <c r="K38" s="79">
+      <c r="L38" s="79">
         <v>4812.0244000000002</v>
       </c>
-      <c r="L38" s="79">
+      <c r="M38" s="79">
         <v>63.037519640000006</v>
       </c>
-      <c r="M38" s="79">
+      <c r="N38" s="79">
         <v>4.1005000000000003</v>
       </c>
-      <c r="N38" s="79">
+      <c r="O38" s="79">
         <v>40</v>
       </c>
-      <c r="O38" s="21">
+      <c r="P38" s="21">
         <v>8.76</v>
       </c>
-      <c r="P38" s="21">
+      <c r="Q38" s="21">
         <v>1</v>
       </c>
-      <c r="T38" s="89" t="s">
+      <c r="U38" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="U38" s="89"/>
-      <c r="V38" s="89" t="str">
+      <c r="V38" s="89"/>
+      <c r="W38" s="89" t="str">
         <f>$B$2&amp;$C$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$16,3)&amp;"_EESTI00"</f>
         <v>ELCTESHL_EESTI00</v>
       </c>
-      <c r="W38" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V38,2)&amp;" Eesti Power plant - Oil Shale"</f>
+      <c r="X38" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W38,2)&amp;" Eesti Power plant - Oil Shale"</f>
         <v>Power Plants Existing00 Eesti Power plant - Oil Shale</v>
       </c>
-      <c r="X38" t="s">
+      <c r="Y38" t="s">
         <v>180</v>
       </c>
-      <c r="Y38" t="s">
+      <c r="Z38" t="s">
         <v>101</v>
       </c>
-      <c r="Z38" t="s">
+      <c r="AA38" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="39" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="39" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B39" s="21" t="str">
-        <f>V39</f>
+        <f>W39</f>
         <v>ELCTESHL_AUVERE00</v>
       </c>
       <c r="C39" s="21" t="str">
@@ -9042,55 +9212,58 @@
       <c r="G39" s="21">
         <v>0.26</v>
       </c>
-      <c r="I39" s="21">
+      <c r="I39" s="7">
+        <v>2</v>
+      </c>
+      <c r="J39" s="21">
         <v>0.33</v>
       </c>
-      <c r="J39" s="21">
+      <c r="K39" s="21">
         <v>0.95</v>
       </c>
-      <c r="K39" s="79">
+      <c r="L39" s="79">
         <v>4812.0244000000002</v>
       </c>
-      <c r="L39" s="79">
+      <c r="M39" s="79">
         <v>63.037519640000006</v>
       </c>
-      <c r="M39" s="79">
+      <c r="N39" s="79">
         <v>4.1005000000000003</v>
       </c>
-      <c r="N39" s="21">
+      <c r="O39" s="21">
         <v>40</v>
       </c>
-      <c r="O39" s="21">
+      <c r="P39" s="21">
         <v>8.76</v>
       </c>
-      <c r="P39" s="21">
+      <c r="Q39" s="21">
         <v>1</v>
       </c>
-      <c r="T39" s="89" t="s">
+      <c r="U39" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="U39" s="89"/>
-      <c r="V39" s="89" t="str">
+      <c r="V39" s="89"/>
+      <c r="W39" s="89" t="str">
         <f>$B$2&amp;$C$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$16,3)&amp;"_AUVERE00"</f>
         <v>ELCTESHL_AUVERE00</v>
       </c>
-      <c r="W39" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V39,2)&amp;" Auvere Power plant - Oil Shale"</f>
+      <c r="X39" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W39,2)&amp;" Auvere Power plant - Oil Shale"</f>
         <v>Power Plants Existing00 Auvere Power plant - Oil Shale</v>
       </c>
-      <c r="X39" t="s">
+      <c r="Y39" t="s">
         <v>180</v>
       </c>
-      <c r="Y39" t="s">
+      <c r="Z39" t="s">
         <v>101</v>
       </c>
-      <c r="Z39" t="s">
+      <c r="AA39" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="40" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B40" s="21" t="str">
-        <f>V40</f>
+        <f>W40</f>
         <v>ELCTESHL_ENEFIT00</v>
       </c>
       <c r="C40" s="21" t="str">
@@ -9104,55 +9277,58 @@
       <c r="G40" s="21">
         <v>0.01</v>
       </c>
-      <c r="I40" s="21">
+      <c r="I40" s="7">
+        <v>2</v>
+      </c>
+      <c r="J40" s="21">
         <v>0.33</v>
       </c>
-      <c r="J40" s="21">
+      <c r="K40" s="21">
         <v>0.95</v>
       </c>
-      <c r="K40" s="79">
+      <c r="L40" s="79">
         <v>4812.0244000000002</v>
       </c>
-      <c r="L40" s="79">
+      <c r="M40" s="79">
         <v>63.037519640000006</v>
       </c>
-      <c r="M40" s="79">
+      <c r="N40" s="79">
         <v>4.1005000000000003</v>
       </c>
-      <c r="N40" s="21">
+      <c r="O40" s="21">
         <v>40</v>
       </c>
-      <c r="O40" s="21">
+      <c r="P40" s="21">
         <v>8.76</v>
       </c>
-      <c r="P40" s="21">
+      <c r="Q40" s="21">
         <v>1</v>
       </c>
-      <c r="T40" s="89" t="s">
+      <c r="U40" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="U40" s="89"/>
-      <c r="V40" s="89" t="str">
+      <c r="V40" s="89"/>
+      <c r="W40" s="89" t="str">
         <f>$B$2&amp;$C$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$16,3)&amp;"_ENEFIT00"</f>
         <v>ELCTESHL_ENEFIT00</v>
       </c>
-      <c r="W40" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V40,2)&amp;" Eenefit Power plant - Oil Shale"</f>
+      <c r="X40" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W40,2)&amp;" Eenefit Power plant - Oil Shale"</f>
         <v>Power Plants Existing00 Eenefit Power plant - Oil Shale</v>
       </c>
-      <c r="X40" t="s">
+      <c r="Y40" t="s">
         <v>180</v>
       </c>
-      <c r="Y40" t="s">
+      <c r="Z40" t="s">
         <v>101</v>
       </c>
-      <c r="Z40" t="s">
+      <c r="AA40" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="41" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="41" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B41" s="21" t="str">
-        <f>V41</f>
+        <f>W41</f>
         <v>ELCTESHL_BALTI00</v>
       </c>
       <c r="C41" s="21" t="str">
@@ -9166,55 +9342,58 @@
       <c r="G41" s="21">
         <v>0.185</v>
       </c>
-      <c r="I41" s="21">
+      <c r="I41" s="7">
+        <v>2</v>
+      </c>
+      <c r="J41" s="21">
         <v>0.33</v>
       </c>
-      <c r="J41" s="21">
+      <c r="K41" s="21">
         <v>0.95</v>
       </c>
-      <c r="K41" s="79">
+      <c r="L41" s="79">
         <v>4812.0244000000002</v>
       </c>
-      <c r="L41" s="79">
+      <c r="M41" s="79">
         <v>63.037519640000006</v>
       </c>
-      <c r="M41" s="79">
+      <c r="N41" s="79">
         <v>4.1005000000000003</v>
       </c>
-      <c r="N41" s="21">
+      <c r="O41" s="21">
         <v>40</v>
       </c>
-      <c r="O41" s="21">
+      <c r="P41" s="21">
         <v>8.76</v>
       </c>
-      <c r="P41" s="21">
+      <c r="Q41" s="21">
         <v>1</v>
       </c>
-      <c r="T41" s="89" t="s">
+      <c r="U41" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="U41" s="89"/>
-      <c r="V41" s="89" t="str">
+      <c r="V41" s="89"/>
+      <c r="W41" s="89" t="str">
         <f>$B$2&amp;$C$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$16,3)&amp;"_BALTI00"</f>
         <v>ELCTESHL_BALTI00</v>
       </c>
-      <c r="W41" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V41,2)&amp;" Balti Power plant - Oil Shale"</f>
+      <c r="X41" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W41,2)&amp;" Balti Power plant - Oil Shale"</f>
         <v>Power Plants Existing00 Balti Power plant - Oil Shale</v>
       </c>
-      <c r="X41" t="s">
+      <c r="Y41" t="s">
         <v>180</v>
       </c>
-      <c r="Y41" t="s">
+      <c r="Z41" t="s">
         <v>101</v>
       </c>
-      <c r="Z41" t="s">
+      <c r="AA41" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="42" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B42" s="21" t="str">
-        <f>V42</f>
+        <f>W42</f>
         <v>ELCTESHL_SILLAMAE00</v>
       </c>
       <c r="C42" s="21" t="str">
@@ -9228,54 +9407,57 @@
       <c r="G42" s="21">
         <v>0.01</v>
       </c>
-      <c r="I42" s="21">
+      <c r="I42" s="7">
+        <v>2</v>
+      </c>
+      <c r="J42" s="21">
         <v>0.33</v>
       </c>
-      <c r="J42" s="21">
+      <c r="K42" s="21">
         <v>0.95</v>
       </c>
-      <c r="K42" s="79">
+      <c r="L42" s="79">
         <v>4812.0244000000002</v>
       </c>
-      <c r="L42" s="79">
+      <c r="M42" s="79">
         <v>63.037519640000006</v>
       </c>
-      <c r="M42" s="79">
+      <c r="N42" s="79">
         <v>4.1005000000000003</v>
       </c>
-      <c r="N42" s="21">
+      <c r="O42" s="21">
         <v>40</v>
       </c>
-      <c r="O42" s="21">
+      <c r="P42" s="21">
         <v>8.76</v>
       </c>
-      <c r="P42" s="21">
+      <c r="Q42" s="21">
         <v>1</v>
       </c>
-      <c r="T42" s="89" t="s">
+      <c r="U42" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V42" s="89" t="str">
+      <c r="W42" s="89" t="str">
         <f>$B$2&amp;$C$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$16,3)&amp;"_SILLAMAE00"</f>
         <v>ELCTESHL_SILLAMAE00</v>
       </c>
-      <c r="W42" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V42,2)&amp;" Sillamae Power plant - Oil Shale"</f>
+      <c r="X42" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W42,2)&amp;" Sillamae Power plant - Oil Shale"</f>
         <v>Power Plants Existing00 Sillamae Power plant - Oil Shale</v>
       </c>
-      <c r="X42" t="s">
+      <c r="Y42" t="s">
         <v>180</v>
       </c>
-      <c r="Y42" t="s">
+      <c r="Z42" t="s">
         <v>101</v>
       </c>
-      <c r="Z42" t="s">
+      <c r="AA42" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="43" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B43" s="21" t="str">
-        <f t="shared" ref="B43:B45" si="3">V43</f>
+        <f t="shared" ref="B43:B45" si="3">W43</f>
         <v>ELCTEGAS_POHJA00</v>
       </c>
       <c r="C43" s="21" t="str">
@@ -9289,53 +9471,56 @@
       <c r="G43" s="21">
         <v>7.6999999999999999E-2</v>
       </c>
-      <c r="I43" s="74">
+      <c r="I43" s="7">
+        <v>2</v>
+      </c>
+      <c r="J43" s="74">
         <v>0.56000000000000005</v>
       </c>
-      <c r="J43" s="21">
+      <c r="K43" s="21">
         <v>0.95</v>
       </c>
-      <c r="K43" s="79">
+      <c r="L43" s="79">
         <v>1175.5066999999999</v>
       </c>
-      <c r="L43" s="79">
+      <c r="M43" s="79">
         <v>39.138495576499992</v>
       </c>
-      <c r="M43" s="79">
+      <c r="N43" s="79">
         <v>5.8775000000000004</v>
       </c>
-      <c r="N43" s="79">
+      <c r="O43" s="79">
         <v>40</v>
       </c>
-      <c r="O43" s="21">
+      <c r="P43" s="21">
         <v>8.76</v>
       </c>
-      <c r="P43" s="21">
+      <c r="Q43" s="21">
         <v>1</v>
       </c>
-      <c r="T43" s="89" t="s">
+      <c r="U43" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="U43" s="89"/>
-      <c r="V43" s="89" t="str">
+      <c r="V43" s="89"/>
+      <c r="W43" s="89" t="str">
         <f>$B$2&amp;$C$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$6,3)&amp;"_POHJA00"</f>
         <v>ELCTEGAS_POHJA00</v>
       </c>
-      <c r="W43" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V43,2)&amp;" Pohja Power plant - "&amp;'EB1'!E3</f>
+      <c r="X43" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W43,2)&amp;" Pohja Power plant - "&amp;'EB1'!E3</f>
         <v>Power Plants Existing00 Pohja Power plant - Natural Gas</v>
       </c>
-      <c r="X43" t="s">
+      <c r="Y43" t="s">
         <v>180</v>
       </c>
-      <c r="Y43" t="s">
+      <c r="Z43" t="s">
         <v>101</v>
       </c>
-      <c r="Z43" t="s">
+      <c r="AA43" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="44" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="44" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B44" s="21" t="str">
         <f t="shared" si="3"/>
         <v>ELCTEBIO_TLNUTILITAS00</v>
@@ -9351,52 +9536,55 @@
       <c r="G44" s="21">
         <v>3.9E-2</v>
       </c>
-      <c r="I44" s="74">
+      <c r="I44" s="7">
+        <v>2</v>
+      </c>
+      <c r="J44" s="74">
         <v>0.46800000000000003</v>
       </c>
-      <c r="J44" s="21">
+      <c r="K44" s="21">
         <v>0.95</v>
       </c>
-      <c r="K44" s="79">
+      <c r="L44" s="79">
         <v>2950.7891</v>
       </c>
-      <c r="L44" s="79">
+      <c r="M44" s="79">
         <v>133.5792717679</v>
       </c>
-      <c r="M44" s="79">
+      <c r="N44" s="79">
         <v>2.8138000000000001</v>
       </c>
-      <c r="N44" s="79">
+      <c r="O44" s="79">
         <v>40</v>
       </c>
-      <c r="O44" s="21">
+      <c r="P44" s="21">
         <v>8.76</v>
       </c>
-      <c r="P44" s="21">
+      <c r="Q44" s="21">
         <v>1</v>
       </c>
-      <c r="T44" s="89" t="s">
+      <c r="U44" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V44" s="89" t="str">
+      <c r="W44" s="89" t="str">
         <f>$B$2&amp;$C$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$9,3)&amp;"_TLNUTILITAS00"</f>
         <v>ELCTEBIO_TLNUTILITAS00</v>
       </c>
-      <c r="W44" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V44,2)&amp;" Tallinn Utilitas Power plant - "&amp;'EB1'!$O$3</f>
+      <c r="X44" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W44,2)&amp;" Tallinn Utilitas Power plant - "&amp;'EB1'!$O$3</f>
         <v>Power Plants Existing00 Tallinn Utilitas Power plant - Biomass</v>
       </c>
-      <c r="X44" t="s">
+      <c r="Y44" t="s">
         <v>180</v>
       </c>
-      <c r="Y44" t="s">
+      <c r="Z44" t="s">
         <v>101</v>
       </c>
-      <c r="Z44" t="s">
+      <c r="AA44" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="45" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="45" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B45" s="21" t="str">
         <f t="shared" si="3"/>
         <v>ELCTEBIO_TARTU00</v>
@@ -9412,54 +9600,57 @@
       <c r="G45" s="21">
         <v>2.2100000000000002E-2</v>
       </c>
-      <c r="I45" s="74">
+      <c r="I45" s="7">
+        <v>2</v>
+      </c>
+      <c r="J45" s="74">
         <v>0.46800000000000003</v>
       </c>
-      <c r="J45" s="21">
+      <c r="K45" s="21">
         <v>0.95</v>
       </c>
-      <c r="K45" s="79">
+      <c r="L45" s="79">
         <v>2950.7891</v>
       </c>
-      <c r="L45" s="79">
+      <c r="M45" s="79">
         <v>133.5792717679</v>
       </c>
-      <c r="M45" s="79">
+      <c r="N45" s="79">
         <v>2.8138000000000001</v>
       </c>
-      <c r="N45" s="79">
+      <c r="O45" s="79">
         <v>40</v>
       </c>
-      <c r="O45" s="21">
+      <c r="P45" s="21">
         <v>8.76</v>
       </c>
-      <c r="P45" s="21">
+      <c r="Q45" s="21">
         <v>1</v>
       </c>
-      <c r="T45" s="89" t="s">
+      <c r="U45" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V45" s="89" t="str">
+      <c r="W45" s="89" t="str">
         <f>$B$2&amp;$C$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$9,3)&amp;"_TARTU00"</f>
         <v>ELCTEBIO_TARTU00</v>
       </c>
-      <c r="W45" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V45,2)&amp;" Tartu Power plant - "&amp;'EB1'!$O$3</f>
+      <c r="X45" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W45,2)&amp;" Tartu Power plant - "&amp;'EB1'!$O$3</f>
         <v>Power Plants Existing00 Tartu Power plant - Biomass</v>
       </c>
-      <c r="X45" t="s">
+      <c r="Y45" t="s">
         <v>180</v>
       </c>
-      <c r="Y45" t="s">
+      <c r="Z45" t="s">
         <v>101</v>
       </c>
-      <c r="Z45" t="s">
+      <c r="AA45" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="46" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="46" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B46" s="21" t="str">
-        <f>V46</f>
+        <f>W46</f>
         <v>ELCTEBIO_PARNU00</v>
       </c>
       <c r="C46" s="21" t="str">
@@ -9473,54 +9664,57 @@
       <c r="G46" s="21">
         <v>2.0500000000000001E-2</v>
       </c>
-      <c r="I46" s="74">
+      <c r="I46" s="7">
+        <v>2</v>
+      </c>
+      <c r="J46" s="74">
         <v>0.46800000000000003</v>
       </c>
-      <c r="J46" s="21">
+      <c r="K46" s="21">
         <v>0.95</v>
       </c>
-      <c r="K46" s="79">
+      <c r="L46" s="79">
         <v>2950.7891</v>
       </c>
-      <c r="L46" s="79">
+      <c r="M46" s="79">
         <v>133.5792717679</v>
       </c>
-      <c r="M46" s="79">
+      <c r="N46" s="79">
         <v>2.8138000000000001</v>
       </c>
-      <c r="N46" s="79">
+      <c r="O46" s="79">
         <v>40</v>
       </c>
-      <c r="O46" s="21">
+      <c r="P46" s="21">
         <v>8.76</v>
       </c>
-      <c r="P46" s="21">
+      <c r="Q46" s="21">
         <v>1</v>
       </c>
-      <c r="T46" s="89" t="s">
+      <c r="U46" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V46" s="89" t="str">
+      <c r="W46" s="89" t="str">
         <f>$B$2&amp;$C$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$9,3)&amp;"_PARNU00"</f>
         <v>ELCTEBIO_PARNU00</v>
       </c>
-      <c r="W46" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V46,2)&amp;" Parnu Power plant - "&amp;'EB1'!$O$3</f>
+      <c r="X46" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W46,2)&amp;" Parnu Power plant - "&amp;'EB1'!$O$3</f>
         <v>Power Plants Existing00 Parnu Power plant - Biomass</v>
       </c>
-      <c r="X46" t="s">
+      <c r="Y46" t="s">
         <v>180</v>
       </c>
-      <c r="Y46" t="s">
+      <c r="Z46" t="s">
         <v>101</v>
       </c>
-      <c r="Z46" t="s">
+      <c r="AA46" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="47" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="47" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B47" s="21" t="str">
-        <f>V47</f>
+        <f>W47</f>
         <v>ELCTEBIO_HORIZON00</v>
       </c>
       <c r="C47" s="21" t="str">
@@ -9534,54 +9728,57 @@
       <c r="G47" s="21">
         <v>1.3900000000000001E-2</v>
       </c>
-      <c r="I47" s="74">
+      <c r="I47" s="7">
+        <v>2</v>
+      </c>
+      <c r="J47" s="74">
         <v>0.46800000000000003</v>
       </c>
-      <c r="J47" s="21">
+      <c r="K47" s="21">
         <v>0.95</v>
       </c>
-      <c r="K47" s="79">
+      <c r="L47" s="79">
         <v>2950.7891</v>
       </c>
-      <c r="L47" s="79">
+      <c r="M47" s="79">
         <v>133.5792717679</v>
       </c>
-      <c r="M47" s="79">
+      <c r="N47" s="79">
         <v>2.8138000000000001</v>
       </c>
-      <c r="N47" s="79">
+      <c r="O47" s="79">
         <v>40</v>
       </c>
-      <c r="O47" s="21">
+      <c r="P47" s="21">
         <v>8.76</v>
       </c>
-      <c r="P47" s="21">
+      <c r="Q47" s="21">
         <v>1</v>
       </c>
-      <c r="T47" s="89" t="s">
+      <c r="U47" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V47" s="89" t="str">
+      <c r="W47" s="89" t="str">
         <f>$B$2&amp;$C$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$9,3)&amp;"_HORIZON00"</f>
         <v>ELCTEBIO_HORIZON00</v>
       </c>
-      <c r="W47" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V47,2)&amp;" Horizon Power plant - "&amp;'EB1'!$O$3</f>
+      <c r="X47" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W47,2)&amp;" Horizon Power plant - "&amp;'EB1'!$O$3</f>
         <v>Power Plants Existing00 Horizon Power plant - Biomass</v>
       </c>
-      <c r="X47" t="s">
+      <c r="Y47" t="s">
         <v>180</v>
       </c>
-      <c r="Y47" t="s">
+      <c r="Z47" t="s">
         <v>101</v>
       </c>
-      <c r="Z47" t="s">
+      <c r="AA47" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="48" spans="2:26" x14ac:dyDescent="0.2">
+    <row r="48" spans="2:27" x14ac:dyDescent="0.2">
       <c r="B48" s="21" t="str">
-        <f>V48</f>
+        <f>W48</f>
         <v>ELCTEGAS_GRUNE00</v>
       </c>
       <c r="C48" s="21" t="str">
@@ -9595,53 +9792,56 @@
       <c r="G48" s="21">
         <v>4.0999999999999995E-3</v>
       </c>
-      <c r="I48">
+      <c r="I48" s="7">
+        <v>2</v>
+      </c>
+      <c r="J48">
         <v>0.56000000000000005</v>
       </c>
-      <c r="J48" s="21">
+      <c r="K48" s="21">
         <v>0.95</v>
       </c>
-      <c r="K48" s="7">
+      <c r="L48" s="7">
         <v>1175.5066999999999</v>
       </c>
-      <c r="L48" s="83">
+      <c r="M48" s="83">
         <v>39.138495576499992</v>
       </c>
-      <c r="M48" s="83">
+      <c r="N48" s="83">
         <v>5.8775000000000004</v>
       </c>
-      <c r="N48">
+      <c r="O48">
         <v>40</v>
       </c>
-      <c r="O48" s="21">
+      <c r="P48" s="21">
         <v>8.76</v>
       </c>
-      <c r="P48" s="21">
+      <c r="Q48" s="21">
         <v>1</v>
       </c>
-      <c r="T48" s="89" t="s">
+      <c r="U48" s="89" t="s">
         <v>102</v>
       </c>
-      <c r="V48" s="89" t="str">
+      <c r="W48" s="89" t="str">
         <f>$B$2&amp;$C$5&amp;$H$2&amp;RIGHT(Sector_Fuels_ELC!$L$6,3)&amp;"_GRUNE00"</f>
         <v>ELCTEGAS_GRUNE00</v>
       </c>
-      <c r="W48" t="str">
-        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(V48,2)&amp;" GRUNE Power plant - "&amp;'EB1'!$E$3</f>
+      <c r="X48" t="str">
+        <f>$D$2&amp;" "&amp;$H$1&amp;RIGHT(W48,2)&amp;" GRUNE Power plant - "&amp;'EB1'!$E$3</f>
         <v>Power Plants Existing00 GRUNE Power plant - Natural Gas</v>
       </c>
-      <c r="X48" t="s">
+      <c r="Y48" t="s">
         <v>180</v>
       </c>
-      <c r="Y48" t="s">
+      <c r="Z48" t="s">
         <v>101</v>
       </c>
-      <c r="Z48" t="s">
+      <c r="AA48" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="65529" spans="19:19" x14ac:dyDescent="0.2">
-      <c r="S65529" s="29"/>
+    <row r="65529" spans="20:20" x14ac:dyDescent="0.2">
+      <c r="T65529" s="29"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10054,7 +10254,7 @@
         <v>ELCBIO</v>
       </c>
       <c r="D12" s="92" t="str">
-        <f>ELC!$V$5</f>
+        <f>ELC!$W$5</f>
         <v>ELC</v>
       </c>
       <c r="E12">
@@ -10122,7 +10322,7 @@
         <v>ELCBIO</v>
       </c>
       <c r="D13" s="92" t="str">
-        <f>ELC!$V$5</f>
+        <f>ELC!$W$5</f>
         <v>ELC</v>
       </c>
       <c r="E13">
@@ -10190,7 +10390,7 @@
         <v>ELCBIO</v>
       </c>
       <c r="D14" s="92" t="str">
-        <f>ELC!$V$5</f>
+        <f>ELC!$W$5</f>
         <v>ELC</v>
       </c>
       <c r="E14">
@@ -10258,7 +10458,7 @@
         <v>ELCGAS</v>
       </c>
       <c r="D15" s="92" t="str">
-        <f>ELC!$V$5</f>
+        <f>ELC!$W$5</f>
         <v>ELC</v>
       </c>
       <c r="E15">
@@ -10326,7 +10526,7 @@
         <v>ELCBIO</v>
       </c>
       <c r="D16" s="92" t="str">
-        <f>ELC!$V$5</f>
+        <f>ELC!$W$5</f>
         <v>ELC</v>
       </c>
       <c r="E16">
@@ -10394,7 +10594,7 @@
         <v>ELCBIO</v>
       </c>
       <c r="D17" s="92" t="str">
-        <f>ELC!$V$5</f>
+        <f>ELC!$W$5</f>
         <v>ELC</v>
       </c>
       <c r="E17">
@@ -10462,7 +10662,7 @@
         <v>ELCBIO</v>
       </c>
       <c r="D18" s="92" t="str">
-        <f>ELC!$V$5</f>
+        <f>ELC!$W$5</f>
         <v>ELC</v>
       </c>
       <c r="E18">
@@ -10530,7 +10730,7 @@
         <v>ELCGAS</v>
       </c>
       <c r="D19" s="92" t="str">
-        <f>ELC!$V$5</f>
+        <f>ELC!$W$5</f>
         <v>ELC</v>
       </c>
       <c r="E19">
@@ -10594,7 +10794,7 @@
         <v>ELCGAS</v>
       </c>
       <c r="D20" s="92" t="str">
-        <f>ELC!$V$5</f>
+        <f>ELC!$W$5</f>
         <v>ELC</v>
       </c>
       <c r="E20">
@@ -10658,7 +10858,7 @@
         <v>ELCBIO</v>
       </c>
       <c r="D21" s="92" t="str">
-        <f>ELC!$V$5</f>
+        <f>ELC!$W$5</f>
         <v>ELC</v>
       </c>
       <c r="E21">
@@ -10722,7 +10922,7 @@
         <v>ELCBIO</v>
       </c>
       <c r="D22" s="92" t="str">
-        <f>ELC!$V$5</f>
+        <f>ELC!$W$5</f>
         <v>ELC</v>
       </c>
       <c r="E22">
@@ -10786,7 +10986,7 @@
         <v>ELCBIO</v>
       </c>
       <c r="D23" s="92" t="str">
-        <f>ELC!$V$5</f>
+        <f>ELC!$W$5</f>
         <v>ELC</v>
       </c>
       <c r="E23">
@@ -10850,7 +11050,7 @@
         <v>ELCBIO</v>
       </c>
       <c r="D24" s="92" t="str">
-        <f>ELC!$V$5</f>
+        <f>ELC!$W$5</f>
         <v>ELC</v>
       </c>
       <c r="E24">
@@ -11210,7 +11410,7 @@
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B8" s="21" t="str">
-        <f>ELC!$V$6</f>
+        <f>ELC!$W$6</f>
         <v>ELCCO2</v>
       </c>
       <c r="C8" s="63">

</xml_diff>

<commit_message>
Attempt: change PASTI~2025 TO PASTI for base PPs
</commit_message>
<xml_diff>
--- a/VT_EE_ELC_V01.xlsx
+++ b/VT_EE_ELC_V01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{792619DC-794A-4EFD-87FE-9336FA30E4FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D08888B1-4F70-40C0-84D5-6BBB844D8B3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="901" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2333,7 +2333,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="616" uniqueCount="211">
   <si>
     <t>CommName</t>
   </si>
@@ -2953,9 +2953,6 @@
     <t>NCAP_BND~0</t>
   </si>
   <si>
-    <t>PASTI~2025</t>
-  </si>
-  <si>
     <t>TWh2PJ</t>
   </si>
   <si>
@@ -2963,6 +2960,12 @@
   </si>
   <si>
     <t>EFF TWh</t>
+  </si>
+  <si>
+    <t>M€2025/TWh</t>
+  </si>
+  <si>
+    <t>PASTI</t>
   </si>
 </sst>
 </file>
@@ -6996,7 +6999,8 @@
     <col min="12" max="12" width="8.140625" style="21" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10" style="21" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="8.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.5703125" style="21" customWidth="1"/>
+    <col min="16" max="16" width="8.85546875" style="21" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="15" style="21" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="13.28515625" style="21" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="2" style="21" bestFit="1" customWidth="1"/>
@@ -7176,7 +7180,7 @@
       <c r="I5" s="9"/>
       <c r="J5" s="9"/>
       <c r="L5" s="21" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="M5" s="9"/>
       <c r="V5" s="85" t="s">
@@ -7274,7 +7278,7 @@
         <v>160</v>
       </c>
       <c r="G9" s="67" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="H9" s="67" t="s">
         <v>144</v>
@@ -7366,10 +7370,10 @@
       </c>
       <c r="I10" s="15"/>
       <c r="J10" s="15" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="K10" s="15" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="L10" s="73" t="s">
         <v>82</v>
@@ -7424,7 +7428,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="2:30" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:30" ht="23.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B11" s="14" t="s">
         <v>76</v>
       </c>
@@ -7458,9 +7462,8 @@
         <f>$G$2&amp;"/"&amp;$F$2</f>
         <v>M€2025/GW</v>
       </c>
-      <c r="O11" s="13" t="str">
-        <f>$G$2&amp;"/"&amp;$E$2</f>
-        <v>M€2025/PJ</v>
+      <c r="O11" s="13" t="s">
+        <v>209</v>
       </c>
       <c r="P11" s="13" t="s">
         <v>77</v>

</xml_diff>

<commit_message>
Changing lifetime of Oil shale plants
</commit_message>
<xml_diff>
--- a/VT_EE_ELC_V01.xlsx
+++ b/VT_EE_ELC_V01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D08888B1-4F70-40C0-84D5-6BBB844D8B3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{569139BA-E0C6-4733-B24E-BDFDD7D95A47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="901" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9236,7 +9236,7 @@
         <v>5.8775000000000004</v>
       </c>
       <c r="P37" s="79">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="Q37" s="21">
         <v>8.76</v>
@@ -9304,7 +9304,7 @@
         <v>4.1005000000000003</v>
       </c>
       <c r="P38" s="79">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="Q38" s="21">
         <v>8.76</v>
@@ -9373,7 +9373,7 @@
         <v>4.1005000000000003</v>
       </c>
       <c r="P39" s="21">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="Q39" s="21">
         <v>8.76</v>
@@ -9442,7 +9442,7 @@
         <v>4.1005000000000003</v>
       </c>
       <c r="P40" s="21">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="Q40" s="21">
         <v>8.76</v>
@@ -9511,7 +9511,7 @@
         <v>4.1005000000000003</v>
       </c>
       <c r="P41" s="21">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="Q41" s="21">
         <v>8.76</v>
@@ -9580,7 +9580,7 @@
         <v>4.1005000000000003</v>
       </c>
       <c r="P42" s="21">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="Q42" s="21">
         <v>8.76</v>

</xml_diff>

<commit_message>
Testing whether emission is in PJ or TWh by adding emission value in kt/TWh on gas (515 kt/TWh) and oil shale (900 kt/TWh)
</commit_message>
<xml_diff>
--- a/VT_EE_ELC_V01.xlsx
+++ b/VT_EE_ELC_V01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{569139BA-E0C6-4733-B24E-BDFDD7D95A47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8ABDFE5-FEB1-4AAD-9D8D-E1F2E6BC29D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="901" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="901" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EB1" sheetId="133" r:id="rId1"/>
@@ -6318,7 +6318,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="2:18" ht="23.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:18" ht="34.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B20" s="15" t="s">
         <v>37</v>
       </c>
@@ -7346,7 +7346,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="2:30" ht="23.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:30" ht="34.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B10" s="15" t="s">
         <v>37</v>
       </c>
@@ -7428,7 +7428,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="2:30" ht="23.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:30" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B11" s="14" t="s">
         <v>76</v>
       </c>
@@ -11594,19 +11594,27 @@
       <c r="C8" s="63">
         <v>95</v>
       </c>
-      <c r="D8" s="63">
-        <v>56.1</v>
+      <c r="D8">
+        <v>515</v>
       </c>
       <c r="E8" s="63">
         <v>76.400000000000006</v>
       </c>
-      <c r="F8" s="63">
-        <v>100</v>
+      <c r="F8">
+        <v>900</v>
       </c>
       <c r="G8" s="63">
         <v>41.4</v>
       </c>
       <c r="H8" s="1"/>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="D9" s="63">
+        <v>56.1</v>
+      </c>
+      <c r="F9" s="63">
+        <v>100</v>
+      </c>
     </row>
     <row r="23" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B23" s="43"/>

</xml_diff>